<commit_message>
taking off hard coded "no data" status
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -79,7 +79,7 @@
     <t xml:space="preserve">Also Show Under Objective</t>
   </si>
   <si>
-    <t xml:space="preserve">Optional. The ID of a Strategic Plan Objective (ob…) to show the same KPI under in the Strategic Plan Goal View as well. For more than one Objective, separate the IDs with commas, such as ob18, ob19. Leave blank if the KPI does not belong under an Objective.</t>
+    <t xml:space="preserve">Optional. The ID of a Strategic Plan Objective (ob…) to show the same KPI under in the Strategic Plan Goal View as well. For more than one Objective, separate the IDs with commas, such as ob18, ob19. The KPI's status then counts toward that Objective's color. Leave blank if the KPI does not belong under an Objective.</t>
   </si>
   <si>
     <t xml:space="preserve">Objective Name (auto)</t>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Drives Status</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes: this KPI sets the color of its Key Service or Program on the dashboard. No: the KPI is shown but does not change any color. Has no effect on Work Systems or Objectives: a Work System always takes its color from its Key Services, and an Objective from the Programs tagged to it.</t>
+    <t xml:space="preserve">Yes: this KPI sets the color of its Key Service or Program on the dashboard. No: the KPI is shown but does not change any color. Has no effect on Work Systems or Objectives: a Work System always takes its color from its Key Services, and an Objective from the Programs tagged to it plus any KPIs shown under it.</t>
   </si>
   <si>
     <t xml:space="preserve">After editing</t>

</xml_diff>

<commit_message>
taking hard code off work system for status too
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="399">
   <si>
     <t xml:space="preserve">KPI tracking workbook</t>
   </si>
@@ -227,9 +227,6 @@
   </si>
   <si>
     <t xml:space="preserve">Benchmark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
   </si>
   <si>
     <t xml:space="preserve">Every 2 years</t>
@@ -2042,17 +2039,17 @@
         <v>15</v>
       </c>
       <c r="N2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="S2" s="2"/>
     </row>
@@ -10163,7 +10160,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8" t="n">
@@ -10173,7 +10170,7 @@
         <v>76.6</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10181,7 +10178,7 @@
         <v>59</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8" t="n">
@@ -10191,7 +10188,7 @@
         <v>75.1</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10199,7 +10196,7 @@
         <v>59</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8" t="n">
@@ -10215,10 +10212,10 @@
         <v>59</v>
       </c>
       <c r="B5" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>75</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>79.9</v>
@@ -10231,10 +10228,10 @@
         <v>59</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>78.2</v>
@@ -18222,33 +18219,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>83</v>
       </c>
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
@@ -18256,13 +18253,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>85</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -18270,13 +18267,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>87</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -18284,13 +18281,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>88</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>89</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
@@ -18298,13 +18295,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
@@ -18312,13 +18309,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>92</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>93</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
@@ -18326,65 +18323,65 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -18396,2506 +18393,2506 @@
         <v>61</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D13" s="10"/>
       <c r="E13" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D14" s="10"/>
       <c r="E14" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D20" s="10"/>
       <c r="E20" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D21" s="10"/>
       <c r="E21" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D22" s="10"/>
       <c r="E22" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D23" s="10"/>
       <c r="E23" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D24" s="10"/>
       <c r="E24" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D25" s="10"/>
       <c r="E25" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D26" s="10"/>
       <c r="E26" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="B27" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="C27" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>133</v>
-      </c>
       <c r="D27" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>135</v>
-      </c>
       <c r="D28" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B29" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C29" s="10" t="s">
-        <v>137</v>
-      </c>
       <c r="D29" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B30" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>139</v>
-      </c>
       <c r="D30" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B31" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>141</v>
-      </c>
       <c r="D31" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F31" s="10"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C32" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B32" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>143</v>
-      </c>
       <c r="D32" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C33" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="B33" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>145</v>
-      </c>
       <c r="D33" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="B34" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>147</v>
-      </c>
       <c r="D34" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C35" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="B35" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>149</v>
-      </c>
       <c r="D35" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C36" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>151</v>
-      </c>
       <c r="D36" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C37" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="B37" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C37" s="10" t="s">
-        <v>153</v>
-      </c>
       <c r="D37" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C38" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="B38" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>155</v>
-      </c>
       <c r="D38" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B39" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>157</v>
-      </c>
       <c r="D39" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C40" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="B40" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>159</v>
-      </c>
       <c r="D40" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C41" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="B41" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>161</v>
-      </c>
       <c r="D41" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C42" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B42" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>163</v>
-      </c>
       <c r="D42" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C43" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="B43" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>165</v>
-      </c>
       <c r="D43" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C44" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="B44" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>167</v>
-      </c>
       <c r="D44" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C45" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="B45" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C45" s="10" t="s">
-        <v>169</v>
-      </c>
       <c r="D45" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C46" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B46" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C46" s="10" t="s">
-        <v>171</v>
-      </c>
       <c r="D46" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C47" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="B47" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C47" s="10" t="s">
-        <v>173</v>
-      </c>
       <c r="D47" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C48" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="B48" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C48" s="10" t="s">
-        <v>175</v>
-      </c>
       <c r="D48" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="B49" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C49" s="10" t="s">
-        <v>177</v>
-      </c>
       <c r="D49" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="B50" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C50" s="10" t="s">
-        <v>179</v>
-      </c>
       <c r="D50" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C51" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="B51" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C51" s="10" t="s">
-        <v>181</v>
-      </c>
       <c r="D51" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C52" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="B52" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C52" s="10" t="s">
-        <v>183</v>
-      </c>
       <c r="D52" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C53" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="B53" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C53" s="10" t="s">
-        <v>185</v>
-      </c>
       <c r="D53" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C54" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="B54" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>187</v>
-      </c>
       <c r="D54" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C55" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="B55" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C55" s="10" t="s">
-        <v>189</v>
-      </c>
       <c r="D55" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C56" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="B56" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C56" s="10" t="s">
-        <v>191</v>
-      </c>
       <c r="D56" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C57" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="B57" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C57" s="10" t="s">
-        <v>193</v>
-      </c>
       <c r="D57" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C58" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="B58" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C58" s="10" t="s">
-        <v>195</v>
-      </c>
       <c r="D58" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C59" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B59" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C59" s="10" t="s">
-        <v>197</v>
-      </c>
       <c r="D59" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B60" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C60" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="B60" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C60" s="10" t="s">
-        <v>199</v>
-      </c>
       <c r="D60" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C61" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="B61" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C61" s="10" t="s">
-        <v>201</v>
-      </c>
       <c r="D61" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B62" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C62" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="B62" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C62" s="10" t="s">
-        <v>203</v>
-      </c>
       <c r="D62" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B63" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="B63" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C63" s="10" t="s">
-        <v>205</v>
-      </c>
       <c r="D63" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="B64" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C64" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="B64" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C64" s="10" t="s">
-        <v>207</v>
-      </c>
       <c r="D64" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="B65" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C65" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="B65" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C65" s="10" t="s">
-        <v>209</v>
-      </c>
       <c r="D65" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B66" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C66" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="B66" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C66" s="10" t="s">
-        <v>211</v>
-      </c>
       <c r="D66" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B67" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C67" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="B67" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C67" s="10" t="s">
-        <v>213</v>
-      </c>
       <c r="D67" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F67" s="10"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="B68" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C68" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="B68" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C68" s="10" t="s">
-        <v>215</v>
-      </c>
       <c r="D68" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="B69" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C69" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="B69" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C69" s="10" t="s">
-        <v>217</v>
-      </c>
       <c r="D69" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F69" s="10"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="B70" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C70" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="B70" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C70" s="10" t="s">
-        <v>219</v>
-      </c>
       <c r="D70" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F70" s="10"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="B71" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C71" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="B71" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C71" s="10" t="s">
-        <v>221</v>
-      </c>
       <c r="D71" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F71" s="10"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B72" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C72" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="B72" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C72" s="10" t="s">
-        <v>223</v>
-      </c>
       <c r="D72" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B73" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C73" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="B73" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C73" s="10" t="s">
-        <v>225</v>
-      </c>
       <c r="D73" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F73" s="10"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="B74" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C74" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="B74" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C74" s="10" t="s">
-        <v>227</v>
-      </c>
       <c r="D74" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B75" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C75" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="B75" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C75" s="10" t="s">
-        <v>229</v>
-      </c>
       <c r="D75" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F75" s="10"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="B76" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C76" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="B76" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C76" s="10" t="s">
-        <v>231</v>
-      </c>
       <c r="D76" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="B77" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C77" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="B77" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C77" s="10" t="s">
-        <v>233</v>
-      </c>
       <c r="D77" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F77" s="10"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B78" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C78" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="B78" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C78" s="10" t="s">
-        <v>235</v>
-      </c>
       <c r="D78" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B79" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C79" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="B79" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C79" s="10" t="s">
-        <v>237</v>
-      </c>
       <c r="D79" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F79" s="10"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B80" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C80" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="B80" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C80" s="10" t="s">
-        <v>239</v>
-      </c>
       <c r="D80" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="B81" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C81" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="B81" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C81" s="10" t="s">
-        <v>241</v>
-      </c>
       <c r="D81" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F81" s="10"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B82" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C82" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="B82" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C82" s="10" t="s">
-        <v>243</v>
-      </c>
       <c r="D82" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="B83" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C83" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="B83" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C83" s="10" t="s">
-        <v>245</v>
-      </c>
       <c r="D83" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F83" s="10"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B84" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C84" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="B84" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C84" s="10" t="s">
-        <v>247</v>
-      </c>
       <c r="D84" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="B85" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C85" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="B85" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C85" s="10" t="s">
-        <v>249</v>
-      </c>
       <c r="D85" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F85" s="10"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="B86" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C86" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="B86" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C86" s="10" t="s">
-        <v>251</v>
-      </c>
       <c r="D86" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="B87" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C87" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="B87" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C87" s="10" t="s">
-        <v>253</v>
-      </c>
       <c r="D87" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F87" s="10"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="B88" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C88" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="B88" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C88" s="10" t="s">
-        <v>255</v>
-      </c>
       <c r="D88" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="B89" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C89" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="B89" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C89" s="10" t="s">
-        <v>257</v>
-      </c>
       <c r="D89" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F89" s="10"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="B90" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C90" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="B90" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C90" s="10" t="s">
-        <v>259</v>
-      </c>
       <c r="D90" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="B91" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C91" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="B91" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C91" s="10" t="s">
-        <v>261</v>
-      </c>
       <c r="D91" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F91" s="10"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="B92" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C92" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="B92" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C92" s="10" t="s">
-        <v>263</v>
-      </c>
       <c r="D92" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="B93" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C93" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="B93" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C93" s="10" t="s">
-        <v>265</v>
-      </c>
       <c r="D93" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F93" s="10"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="B95" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C95" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="B95" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C95" s="10" t="s">
-        <v>268</v>
-      </c>
       <c r="D95" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F95" s="10"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="B96" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C96" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="B96" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C96" s="10" t="s">
-        <v>270</v>
-      </c>
       <c r="D96" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="B97" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C97" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="B97" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C97" s="10" t="s">
-        <v>272</v>
-      </c>
       <c r="D97" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F97" s="10"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="B98" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C98" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="B98" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C98" s="10" t="s">
-        <v>274</v>
-      </c>
       <c r="D98" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B99" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C99" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="B99" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C99" s="10" t="s">
-        <v>276</v>
-      </c>
       <c r="D99" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F99" s="10"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="B100" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C100" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="B100" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C100" s="10" t="s">
-        <v>278</v>
-      </c>
       <c r="D100" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E100" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="B101" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C101" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="B101" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C101" s="10" t="s">
-        <v>280</v>
-      </c>
       <c r="D101" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F101" s="10"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="B102" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C102" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="B102" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C102" s="10" t="s">
-        <v>282</v>
-      </c>
       <c r="D102" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="B103" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C103" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="B103" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C103" s="10" t="s">
-        <v>284</v>
-      </c>
       <c r="D103" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F103" s="10"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="B104" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C104" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="B104" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C104" s="10" t="s">
-        <v>286</v>
-      </c>
       <c r="D104" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E104" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="B105" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C105" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="B105" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C105" s="10" t="s">
-        <v>288</v>
-      </c>
       <c r="D105" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F105" s="10"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="B106" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C106" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="B106" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C106" s="10" t="s">
-        <v>290</v>
-      </c>
       <c r="D106" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E106" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="B107" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C107" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="B107" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C107" s="10" t="s">
-        <v>292</v>
-      </c>
       <c r="D107" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F107" s="10"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="B108" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C108" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="B108" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C108" s="10" t="s">
-        <v>294</v>
-      </c>
       <c r="D108" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E108" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="B109" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C109" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="B109" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C109" s="10" t="s">
-        <v>296</v>
-      </c>
       <c r="D109" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F109" s="10"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="B110" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C110" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="B110" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C110" s="10" t="s">
-        <v>298</v>
-      </c>
       <c r="D110" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E110" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="B111" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C111" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="B111" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C111" s="10" t="s">
-        <v>300</v>
-      </c>
       <c r="D111" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F111" s="10"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="B112" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C112" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="B112" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C112" s="10" t="s">
-        <v>302</v>
-      </c>
       <c r="D112" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E112" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="B113" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C113" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="B113" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C113" s="10" t="s">
-        <v>304</v>
-      </c>
       <c r="D113" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F113" s="10"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="B114" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C114" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="B114" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C114" s="10" t="s">
-        <v>306</v>
-      </c>
       <c r="D114" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E114" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="B115" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C115" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="B115" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C115" s="10" t="s">
-        <v>308</v>
-      </c>
       <c r="D115" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F115" s="10"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="B116" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C116" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="B116" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C116" s="10" t="s">
-        <v>310</v>
-      </c>
       <c r="D116" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E116" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="B117" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C117" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="B117" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C117" s="10" t="s">
-        <v>312</v>
-      </c>
       <c r="D117" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F117" s="10"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="B118" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C118" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="B118" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C118" s="10" t="s">
-        <v>314</v>
-      </c>
       <c r="D118" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E118" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="10" t="s">
+        <v>314</v>
+      </c>
+      <c r="B119" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C119" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="B119" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C119" s="10" t="s">
-        <v>316</v>
-      </c>
       <c r="D119" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F119" s="10"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="B120" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C120" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="B120" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C120" s="10" t="s">
-        <v>318</v>
-      </c>
       <c r="D120" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E120" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="B121" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C121" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="B121" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C121" s="10" t="s">
-        <v>320</v>
-      </c>
       <c r="D121" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E121" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F121" s="10"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="B122" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C122" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="B122" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C122" s="10" t="s">
-        <v>322</v>
-      </c>
       <c r="D122" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E122" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="B123" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C123" s="10" t="s">
         <v>323</v>
       </c>
-      <c r="B123" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C123" s="10" t="s">
-        <v>324</v>
-      </c>
       <c r="D123" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E123" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F123" s="10"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="B124" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C124" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B124" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C124" s="10" t="s">
-        <v>326</v>
-      </c>
       <c r="D124" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E124" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="B125" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C125" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="B125" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C125" s="10" t="s">
-        <v>328</v>
-      </c>
       <c r="D125" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E125" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F125" s="10"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="B126" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C126" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="B126" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C126" s="10" t="s">
-        <v>330</v>
-      </c>
       <c r="D126" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E126" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="B127" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C127" s="10" t="s">
         <v>331</v>
       </c>
-      <c r="B127" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C127" s="10" t="s">
-        <v>332</v>
-      </c>
       <c r="D127" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F127" s="10"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="B128" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C128" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="B128" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C128" s="10" t="s">
-        <v>334</v>
-      </c>
       <c r="D128" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E128" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="B129" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C129" s="10" t="s">
         <v>335</v>
       </c>
-      <c r="B129" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C129" s="10" t="s">
-        <v>336</v>
-      </c>
       <c r="D129" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F129" s="10"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="B130" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C130" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="B130" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C130" s="10" t="s">
-        <v>338</v>
-      </c>
       <c r="D130" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E130" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="B131" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C131" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="B131" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C131" s="10" t="s">
-        <v>340</v>
-      </c>
       <c r="D131" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F131" s="10"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="B132" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C132" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="B132" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C132" s="10" t="s">
-        <v>342</v>
-      </c>
       <c r="D132" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="B133" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C133" s="10" t="s">
         <v>343</v>
       </c>
-      <c r="B133" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C133" s="10" t="s">
-        <v>344</v>
-      </c>
       <c r="D133" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F133" s="10"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="B134" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C134" s="10" t="s">
         <v>345</v>
       </c>
-      <c r="B134" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C134" s="10" t="s">
-        <v>346</v>
-      </c>
       <c r="D134" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E134" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="B135" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C135" s="10" t="s">
         <v>347</v>
       </c>
-      <c r="B135" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C135" s="10" t="s">
-        <v>348</v>
-      </c>
       <c r="D135" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E135" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F135" s="10"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="B136" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C136" s="10" t="s">
         <v>349</v>
       </c>
-      <c r="B136" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C136" s="10" t="s">
-        <v>350</v>
-      </c>
       <c r="D136" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E136" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="10" t="s">
+        <v>350</v>
+      </c>
+      <c r="B137" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C137" s="10" t="s">
         <v>351</v>
       </c>
-      <c r="B137" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C137" s="10" t="s">
-        <v>352</v>
-      </c>
       <c r="D137" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F137" s="10"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="B138" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="B138" s="10" t="s">
+      <c r="C138" s="10" t="s">
         <v>354</v>
-      </c>
-      <c r="C138" s="10" t="s">
-        <v>355</v>
       </c>
       <c r="D138" s="10"/>
       <c r="E138" s="10"/>
       <c r="F138" s="10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="B139" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C139" s="10" t="s">
         <v>357</v>
-      </c>
-      <c r="B139" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C139" s="10" t="s">
-        <v>358</v>
       </c>
       <c r="D139" s="10"/>
       <c r="E139" s="10"/>
       <c r="F139" s="10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="B140" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C140" s="10" t="s">
         <v>359</v>
-      </c>
-      <c r="B140" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C140" s="10" t="s">
-        <v>360</v>
       </c>
       <c r="D140" s="10"/>
       <c r="E140" s="10"/>
       <c r="F140" s="10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="B141" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C141" s="10" t="s">
         <v>361</v>
-      </c>
-      <c r="B141" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C141" s="10" t="s">
-        <v>362</v>
       </c>
       <c r="D141" s="10"/>
       <c r="E141" s="10"/>
       <c r="F141" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="B142" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C142" s="10" t="s">
         <v>364</v>
-      </c>
-      <c r="B142" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C142" s="10" t="s">
-        <v>365</v>
       </c>
       <c r="D142" s="10"/>
       <c r="E142" s="10"/>
       <c r="F142" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="B143" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C143" s="10" t="s">
         <v>366</v>
-      </c>
-      <c r="B143" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C143" s="10" t="s">
-        <v>367</v>
       </c>
       <c r="D143" s="10"/>
       <c r="E143" s="10"/>
       <c r="F143" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="B144" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C144" s="10" t="s">
         <v>368</v>
-      </c>
-      <c r="B144" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C144" s="10" t="s">
-        <v>369</v>
       </c>
       <c r="D144" s="10"/>
       <c r="E144" s="10"/>
       <c r="F144" s="10" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="B145" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C145" s="10" t="s">
         <v>371</v>
-      </c>
-      <c r="B145" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C145" s="10" t="s">
-        <v>372</v>
       </c>
       <c r="D145" s="10"/>
       <c r="E145" s="10"/>
       <c r="F145" s="10" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="10" t="s">
+        <v>372</v>
+      </c>
+      <c r="B146" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C146" s="10" t="s">
         <v>373</v>
-      </c>
-      <c r="B146" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C146" s="10" t="s">
-        <v>374</v>
       </c>
       <c r="D146" s="10"/>
       <c r="E146" s="10"/>
       <c r="F146" s="10" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="B147" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C147" s="10" t="s">
         <v>375</v>
-      </c>
-      <c r="B147" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C147" s="10" t="s">
-        <v>376</v>
       </c>
       <c r="D147" s="10"/>
       <c r="E147" s="10"/>
       <c r="F147" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="10" t="s">
+        <v>377</v>
+      </c>
+      <c r="B148" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C148" s="10" t="s">
         <v>378</v>
-      </c>
-      <c r="B148" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C148" s="10" t="s">
-        <v>379</v>
       </c>
       <c r="D148" s="10"/>
       <c r="E148" s="10"/>
       <c r="F148" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="10" t="s">
+        <v>379</v>
+      </c>
+      <c r="B149" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C149" s="10" t="s">
         <v>380</v>
-      </c>
-      <c r="B149" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C149" s="10" t="s">
-        <v>381</v>
       </c>
       <c r="D149" s="10"/>
       <c r="E149" s="10"/>
       <c r="F149" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="B150" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C150" s="10" t="s">
         <v>382</v>
-      </c>
-      <c r="B150" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C150" s="10" t="s">
-        <v>383</v>
       </c>
       <c r="D150" s="10"/>
       <c r="E150" s="10"/>
       <c r="F150" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="B151" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C151" s="10" t="s">
         <v>384</v>
-      </c>
-      <c r="B151" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C151" s="10" t="s">
-        <v>385</v>
       </c>
       <c r="D151" s="10"/>
       <c r="E151" s="10"/>
       <c r="F151" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="10" t="s">
+        <v>385</v>
+      </c>
+      <c r="B152" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C152" s="10" t="s">
         <v>386</v>
-      </c>
-      <c r="B152" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C152" s="10" t="s">
-        <v>387</v>
       </c>
       <c r="D152" s="10"/>
       <c r="E152" s="10"/>
       <c r="F152" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="B153" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C153" s="10" t="s">
         <v>388</v>
-      </c>
-      <c r="B153" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C153" s="10" t="s">
-        <v>389</v>
       </c>
       <c r="D153" s="10"/>
       <c r="E153" s="10"/>
       <c r="F153" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="B154" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C154" s="10" t="s">
         <v>391</v>
-      </c>
-      <c r="B154" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C154" s="10" t="s">
-        <v>392</v>
       </c>
       <c r="D154" s="10"/>
       <c r="E154" s="10"/>
       <c r="F154" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20903,52 +20900,52 @@
         <v>63</v>
       </c>
       <c r="B155" s="10" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C155" s="10" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D155" s="10"/>
       <c r="E155" s="10"/>
       <c r="F155" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="10" t="s">
+        <v>394</v>
+      </c>
+      <c r="B156" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C156" s="10" t="s">
         <v>395</v>
-      </c>
-      <c r="B156" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C156" s="10" t="s">
-        <v>396</v>
       </c>
       <c r="D156" s="10"/>
       <c r="E156" s="10"/>
       <c r="F156" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="B157" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C157" s="10" t="s">
         <v>397</v>
-      </c>
-      <c r="B157" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="C157" s="10" t="s">
-        <v>398</v>
       </c>
       <c r="D157" s="10"/>
       <c r="E157" s="10"/>
       <c r="F157" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pio social rates added
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/MaryCathryn.Lord/Desktop/CoD_PerformanceDash_External/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA953B49-6729-BF4B-B7E4-10DD7F60519E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62575A8D-B11C-F549-885B-6D3F8BDEAEF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15160" yWindow="660" windowWidth="15080" windowHeight="18980" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15580" yWindow="660" windowWidth="14660" windowHeight="18980" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1183" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="523">
   <si>
     <t>KPI tracking workbook</t>
   </si>
@@ -1587,6 +1587,30 @@
   </si>
   <si>
     <t>Job clickthrough rate</t>
+  </si>
+  <si>
+    <t>PIO-ENGRATE</t>
+  </si>
+  <si>
+    <t>Social media engagement rate</t>
+  </si>
+  <si>
+    <t>Public Information Officer</t>
+  </si>
+  <si>
+    <t>Instagram</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>TikTok</t>
+  </si>
+  <si>
+    <t>Instagram, Facebook, LinkedIn, TikTok</t>
   </si>
 </sst>
 </file>
@@ -3732,7 +3756,7 @@
       <c r="R37" s="2"/>
       <c r="S37" s="2"/>
     </row>
-    <row r="38" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
         <v>490</v>
       </c>
@@ -3756,27 +3780,55 @@
         <f>IF(F38="","",IF(ISNUMBER(SEARCH(",",F38)),"Several items (the script lists them)",IFERROR(INDEX('Dashboard Items'!$B$2:$B$500,MATCH(F38,'Dashboard Items'!$A$2:$A$500,0))&amp;": "&amp;INDEX('Dashboard Items'!$C$2:$C$500,MATCH(F38,'Dashboard Items'!$A$2:$A$500,0)),"ID not found")))</f>
         <v>Key Service: Municipal Court</v>
       </c>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
-      <c r="P38" s="2"/>
-      <c r="Q38" s="2"/>
+      <c r="H38" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I38" s="2">
+        <v>2</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L38" s="2">
+        <v>5</v>
+      </c>
+      <c r="M38" s="2">
+        <v>15</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O38" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="P38" s="12" t="s">
+        <v>517</v>
+      </c>
+      <c r="Q38" s="12" t="s">
+        <v>522</v>
+      </c>
       <c r="R38" s="2"/>
       <c r="S38" s="2"/>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="A39" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>516</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>159</v>
+      </c>
       <c r="E39" s="6" t="str">
         <f>IF(D39="","",IFERROR(IF(INDEX('Dashboard Items'!$B$2:$B$500,MATCH(D39,'Dashboard Items'!$A$2:$A$500,0))="Objective","Objectives go in the next column",IF(OR(C39="",INDEX('Dashboard Items'!$B$2:$B$500,MATCH(D39,'Dashboard Items'!$A$2:$A$500,0))=C39),INDEX('Dashboard Items'!$C$2:$C$500,MATCH(D39,'Dashboard Items'!$A$2:$A$500,0)),"Level does not match ID")),"ID not found"))</f>
-        <v/>
+        <v>Public Outreach</v>
       </c>
       <c r="F39" s="7"/>
       <c r="G39" s="6" t="str">
@@ -11162,7 +11214,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G996"/>
+  <dimension ref="A1:G995"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -12406,156 +12458,360 @@
       <c r="G70" s="2"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A71" s="8"/>
-      <c r="B71" s="9"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="8"/>
-      <c r="E71" s="8"/>
-      <c r="F71" s="8"/>
+      <c r="A71" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B71" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C71" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="D71" s="8">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="E71" s="8">
+        <v>5.9</v>
+      </c>
+      <c r="F71" s="8">
+        <v>2.6</v>
+      </c>
       <c r="G71" s="2"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A72" s="8"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="8"/>
-      <c r="E72" s="8"/>
-      <c r="F72" s="8"/>
+      <c r="A72" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B72" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C72" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="D72" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="E72" s="8">
+        <v>5.9</v>
+      </c>
+      <c r="F72" s="8">
+        <v>2.6</v>
+      </c>
       <c r="G72" s="2"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A73" s="8"/>
-      <c r="B73" s="9"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="8"/>
-      <c r="E73" s="8"/>
-      <c r="F73" s="8"/>
+      <c r="A73" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B73" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C73" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="D73" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E73" s="8">
+        <v>5.9</v>
+      </c>
+      <c r="F73" s="8">
+        <v>2.6</v>
+      </c>
       <c r="G73" s="2"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A74" s="8"/>
-      <c r="B74" s="9"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="8"/>
-      <c r="E74" s="8"/>
-      <c r="F74" s="8"/>
+      <c r="A74" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B74" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C74" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="D74" s="8">
+        <v>5.7</v>
+      </c>
+      <c r="E74" s="8">
+        <v>5.9</v>
+      </c>
+      <c r="F74" s="8">
+        <v>2.6</v>
+      </c>
       <c r="G74" s="2"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A75" s="8"/>
-      <c r="B75" s="9"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
-      <c r="E75" s="8"/>
-      <c r="F75" s="8"/>
+      <c r="A75" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B75" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C75" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="D75" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E75" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="F75" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G75" s="2"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A76" s="8"/>
-      <c r="B76" s="9"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
-      <c r="F76" s="8"/>
+      <c r="A76" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B76" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C76" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="D76" s="8">
+        <v>8.4</v>
+      </c>
+      <c r="E76" s="8">
+        <v>6.5</v>
+      </c>
+      <c r="F76" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G76" s="2"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A77" s="8"/>
-      <c r="B77" s="9"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="8"/>
-      <c r="E77" s="8"/>
-      <c r="F77" s="8"/>
+      <c r="A77" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B77" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C77" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="D77" s="8">
+        <v>6.9</v>
+      </c>
+      <c r="E77" s="8">
+        <v>6.5</v>
+      </c>
+      <c r="F77" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G77" s="2"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A78" s="8"/>
-      <c r="B78" s="9"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="8"/>
-      <c r="E78" s="8"/>
-      <c r="F78" s="8"/>
+      <c r="A78" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B78" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="D78" s="8">
+        <v>7.7</v>
+      </c>
+      <c r="E78" s="8">
+        <v>6.5</v>
+      </c>
+      <c r="F78" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G78" s="2"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A79" s="8"/>
-      <c r="B79" s="9"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="8"/>
-      <c r="F79" s="8"/>
+      <c r="A79" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B79" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C79" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="D79" s="8">
+        <v>6.3</v>
+      </c>
+      <c r="E79" s="8">
+        <v>6.5</v>
+      </c>
+      <c r="F79" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G79" s="2"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A80" s="8"/>
-      <c r="B80" s="9"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="8"/>
-      <c r="E80" s="8"/>
-      <c r="F80" s="8"/>
+      <c r="A80" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B80" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C80" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="D80" s="8">
+        <v>7.9</v>
+      </c>
+      <c r="E80" s="8">
+        <v>6.5</v>
+      </c>
+      <c r="F80" s="8">
+        <v>3.2</v>
+      </c>
       <c r="G80" s="2"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A81" s="8"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="8"/>
-      <c r="E81" s="8"/>
-      <c r="F81" s="8"/>
+      <c r="A81" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B81" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C81" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="D81" s="8">
+        <v>8</v>
+      </c>
+      <c r="E81" s="8">
+        <v>21.2</v>
+      </c>
+      <c r="F81" s="8">
+        <v>2.7</v>
+      </c>
       <c r="G81" s="2"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A82" s="8"/>
-      <c r="B82" s="9"/>
-      <c r="C82" s="8"/>
-      <c r="D82" s="8"/>
-      <c r="E82" s="8"/>
-      <c r="F82" s="8"/>
+      <c r="A82" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B82" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C82" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="D82" s="8">
+        <v>16.8</v>
+      </c>
+      <c r="E82" s="8">
+        <v>21.2</v>
+      </c>
+      <c r="F82" s="8">
+        <v>2.7</v>
+      </c>
       <c r="G82" s="2"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A83" s="8"/>
-      <c r="B83" s="9"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="8"/>
-      <c r="E83" s="8"/>
-      <c r="F83" s="8"/>
+      <c r="A83" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B83" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C83" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="D83" s="8">
+        <v>20.6</v>
+      </c>
+      <c r="E83" s="8">
+        <v>21.2</v>
+      </c>
+      <c r="F83" s="8">
+        <v>2.7</v>
+      </c>
       <c r="G83" s="2"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A84" s="8"/>
-      <c r="B84" s="9"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
+      <c r="A84" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B84" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C84" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="D84" s="8">
+        <v>14.34</v>
+      </c>
+      <c r="E84" s="8">
+        <v>21.2</v>
+      </c>
+      <c r="F84" s="8">
+        <v>3.1</v>
+      </c>
       <c r="G84" s="2"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A85" s="8"/>
-      <c r="B85" s="9"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="8"/>
-      <c r="E85" s="8"/>
-      <c r="F85" s="8"/>
+      <c r="A85" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B85" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C85" s="15" t="s">
+        <v>521</v>
+      </c>
+      <c r="D85" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="E85" s="8">
+        <v>4.7</v>
+      </c>
+      <c r="F85" s="8">
+        <v>1.6</v>
+      </c>
       <c r="G85" s="2"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A86" s="8"/>
-      <c r="B86" s="9"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="8"/>
-      <c r="E86" s="8"/>
-      <c r="F86" s="8"/>
+      <c r="A86" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B86" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C86" s="15" t="s">
+        <v>521</v>
+      </c>
+      <c r="D86" s="8">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="E86" s="8">
+        <v>4.7</v>
+      </c>
+      <c r="F86" s="8">
+        <v>1.6</v>
+      </c>
       <c r="G86" s="2"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A87" s="8"/>
-      <c r="B87" s="9"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="8"/>
-      <c r="E87" s="8"/>
-      <c r="F87" s="8"/>
+      <c r="A87" s="12" t="s">
+        <v>515</v>
+      </c>
+      <c r="B87" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C87" s="15" t="s">
+        <v>521</v>
+      </c>
+      <c r="D87" s="8">
+        <v>5.4</v>
+      </c>
+      <c r="E87" s="8">
+        <v>4.7</v>
+      </c>
+      <c r="F87" s="8">
+        <v>1.6</v>
+      </c>
       <c r="G87" s="2"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
@@ -20729,15 +20985,6 @@
       <c r="E995" s="8"/>
       <c r="F995" s="8"/>
       <c r="G995" s="2"/>
-    </row>
-    <row r="996" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A996" s="8"/>
-      <c r="B996" s="9"/>
-      <c r="C996" s="8"/>
-      <c r="D996" s="8"/>
-      <c r="E996" s="8"/>
-      <c r="F996" s="8"/>
-      <c r="G996" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
library data change to see how it looks
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/MaryCathryn.Lord/Desktop/CoD_PerformanceDash_External/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B954BF5D-F4E6-D54E-950F-30B9B3C1D474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC532635-3796-C94F-BAEF-8580074E06FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71100" yWindow="-7380" windowWidth="30240" windowHeight="19000" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1322" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="510">
   <si>
     <t>KPI tracking workbook</t>
   </si>
@@ -11369,7 +11369,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G1002"/>
+  <dimension ref="A1:G997"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -12864,15 +12864,17 @@
       <c r="B82" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="C82" s="49"/>
+      <c r="C82" s="51" t="s">
+        <v>507</v>
+      </c>
       <c r="D82" s="49">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="E82" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F82" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G82" s="30"/>
     </row>
@@ -12883,15 +12885,17 @@
       <c r="B83" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="C83" s="49"/>
+      <c r="C83" s="51" t="s">
+        <v>507</v>
+      </c>
       <c r="D83" s="49">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="E83" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F83" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G83" s="30"/>
     </row>
@@ -12902,15 +12906,17 @@
       <c r="B84" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="C84" s="49"/>
+      <c r="C84" s="51" t="s">
+        <v>507</v>
+      </c>
       <c r="D84" s="49">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="E84" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F84" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G84" s="30"/>
     </row>
@@ -12921,15 +12927,17 @@
       <c r="B85" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="C85" s="49"/>
+      <c r="C85" s="51" t="s">
+        <v>507</v>
+      </c>
       <c r="D85" s="49">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="E85" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F85" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G85" s="30"/>
     </row>
@@ -12940,15 +12948,17 @@
       <c r="B86" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="C86" s="49"/>
+      <c r="C86" s="51" t="s">
+        <v>507</v>
+      </c>
       <c r="D86" s="49">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="E86" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F86" s="49">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G86" s="30"/>
     </row>
@@ -12960,10 +12970,10 @@
         <v>84</v>
       </c>
       <c r="C87" s="51" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D87" s="49">
-        <v>50</v>
+        <v>88</v>
       </c>
       <c r="E87" s="49">
         <v>50</v>
@@ -12981,10 +12991,10 @@
         <v>77</v>
       </c>
       <c r="C88" s="51" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D88" s="49">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="E88" s="49">
         <v>50</v>
@@ -13002,10 +13012,10 @@
         <v>85</v>
       </c>
       <c r="C89" s="51" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D89" s="49">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="E89" s="49">
         <v>50</v>
@@ -13023,10 +13033,10 @@
         <v>79</v>
       </c>
       <c r="C90" s="51" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D90" s="49">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E90" s="49">
         <v>50</v>
@@ -13044,10 +13054,10 @@
         <v>86</v>
       </c>
       <c r="C91" s="51" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D91" s="49">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="E91" s="49">
         <v>50</v>
@@ -13059,112 +13069,72 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" s="28" t="s">
-        <v>509</v>
-      </c>
-      <c r="B92" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="C92" s="51" t="s">
-        <v>508</v>
-      </c>
-      <c r="D92" s="49">
-        <v>50</v>
-      </c>
-      <c r="E92" s="49">
-        <v>50</v>
-      </c>
-      <c r="F92" s="49">
-        <v>50</v>
-      </c>
+        <v>453</v>
+      </c>
+      <c r="B92" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C92" s="49"/>
+      <c r="D92" s="49"/>
+      <c r="E92" s="49"/>
+      <c r="F92" s="49"/>
       <c r="G92" s="30"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" s="28" t="s">
-        <v>509</v>
-      </c>
-      <c r="B93" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="C93" s="51" t="s">
-        <v>508</v>
-      </c>
-      <c r="D93" s="49">
-        <v>50</v>
-      </c>
-      <c r="E93" s="49">
-        <v>50</v>
-      </c>
-      <c r="F93" s="49">
-        <v>50</v>
-      </c>
+        <v>506</v>
+      </c>
+      <c r="B93" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C93" s="49"/>
+      <c r="D93" s="49"/>
+      <c r="E93" s="49"/>
+      <c r="F93" s="49"/>
       <c r="G93" s="30"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" s="28" t="s">
-        <v>509</v>
-      </c>
-      <c r="B94" s="50" t="s">
-        <v>85</v>
-      </c>
-      <c r="C94" s="51" t="s">
-        <v>508</v>
-      </c>
-      <c r="D94" s="49">
-        <v>50</v>
-      </c>
-      <c r="E94" s="49">
-        <v>50</v>
-      </c>
-      <c r="F94" s="49">
-        <v>50</v>
-      </c>
+        <v>454</v>
+      </c>
+      <c r="B94" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C94" s="49"/>
+      <c r="D94" s="49"/>
+      <c r="E94" s="49"/>
+      <c r="F94" s="49"/>
       <c r="G94" s="30"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" s="28" t="s">
-        <v>509</v>
-      </c>
-      <c r="B95" s="50" t="s">
-        <v>79</v>
-      </c>
-      <c r="C95" s="51" t="s">
-        <v>508</v>
-      </c>
-      <c r="D95" s="49">
-        <v>50</v>
-      </c>
-      <c r="E95" s="49">
-        <v>50</v>
-      </c>
-      <c r="F95" s="49">
-        <v>50</v>
-      </c>
+        <v>455</v>
+      </c>
+      <c r="B95" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C95" s="49"/>
+      <c r="D95" s="49"/>
+      <c r="E95" s="49"/>
+      <c r="F95" s="49"/>
       <c r="G95" s="30"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" s="28" t="s">
-        <v>509</v>
-      </c>
-      <c r="B96" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="C96" s="51" t="s">
-        <v>508</v>
-      </c>
-      <c r="D96" s="49">
-        <v>50</v>
-      </c>
-      <c r="E96" s="49">
-        <v>50</v>
-      </c>
-      <c r="F96" s="49">
-        <v>50</v>
-      </c>
+        <v>456</v>
+      </c>
+      <c r="B96" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C96" s="49"/>
+      <c r="D96" s="49"/>
+      <c r="E96" s="49"/>
+      <c r="F96" s="49"/>
       <c r="G96" s="30"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" s="28" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="B97" s="49" t="s">
         <v>489</v>
@@ -13177,7 +13147,7 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" s="28" t="s">
-        <v>506</v>
+        <v>458</v>
       </c>
       <c r="B98" s="49" t="s">
         <v>489</v>
@@ -13190,182 +13160,162 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" s="28" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B99" s="49" t="s">
-        <v>489</v>
-      </c>
-      <c r="C99" s="49"/>
-      <c r="D99" s="49"/>
-      <c r="E99" s="49"/>
-      <c r="F99" s="49"/>
+        <v>83</v>
+      </c>
+      <c r="C99" s="33"/>
+      <c r="D99" s="49">
+        <v>65014</v>
+      </c>
+      <c r="E99" s="49">
+        <v>71834</v>
+      </c>
+      <c r="F99" s="49">
+        <v>62464</v>
+      </c>
       <c r="G99" s="30"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" s="28" t="s">
-        <v>455</v>
-      </c>
-      <c r="B100" s="49" t="s">
-        <v>489</v>
-      </c>
-      <c r="C100" s="49"/>
-      <c r="D100" s="49"/>
-      <c r="E100" s="49"/>
-      <c r="F100" s="49"/>
+        <v>452</v>
+      </c>
+      <c r="B100" s="50" t="s">
+        <v>84</v>
+      </c>
+      <c r="C100" s="33"/>
+      <c r="D100" s="49">
+        <v>103774</v>
+      </c>
+      <c r="E100" s="49">
+        <v>102033</v>
+      </c>
+      <c r="F100" s="49">
+        <v>88724</v>
+      </c>
       <c r="G100" s="30"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" s="28" t="s">
-        <v>456</v>
-      </c>
-      <c r="B101" s="49" t="s">
-        <v>489</v>
+        <v>452</v>
+      </c>
+      <c r="B101" s="50" t="s">
+        <v>77</v>
       </c>
       <c r="C101" s="49"/>
-      <c r="D101" s="49"/>
-      <c r="E101" s="49"/>
-      <c r="F101" s="49"/>
+      <c r="D101" s="49">
+        <v>211580</v>
+      </c>
+      <c r="E101" s="49">
+        <v>150513</v>
+      </c>
+      <c r="F101" s="49">
+        <v>130881</v>
+      </c>
       <c r="G101" s="30"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" s="28" t="s">
-        <v>457</v>
-      </c>
-      <c r="B102" s="49" t="s">
-        <v>489</v>
+        <v>452</v>
+      </c>
+      <c r="B102" s="50" t="s">
+        <v>85</v>
       </c>
       <c r="C102" s="49"/>
-      <c r="D102" s="49"/>
-      <c r="E102" s="49"/>
-      <c r="F102" s="49"/>
+      <c r="D102" s="49">
+        <v>280116</v>
+      </c>
+      <c r="E102" s="49">
+        <v>173234</v>
+      </c>
+      <c r="F102" s="49">
+        <v>150638</v>
+      </c>
       <c r="G102" s="30"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" s="28" t="s">
-        <v>458</v>
-      </c>
-      <c r="B103" s="49" t="s">
-        <v>489</v>
+        <v>452</v>
+      </c>
+      <c r="B103" s="50" t="s">
+        <v>79</v>
       </c>
       <c r="C103" s="49"/>
-      <c r="D103" s="49"/>
-      <c r="E103" s="49"/>
-      <c r="F103" s="49"/>
+      <c r="D103" s="49">
+        <v>287958</v>
+      </c>
+      <c r="E103" s="49">
+        <v>197111</v>
+      </c>
+      <c r="F103" s="33">
+        <v>171401</v>
+      </c>
       <c r="G103" s="30"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" s="28" t="s">
         <v>452</v>
       </c>
-      <c r="B104" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="C104" s="33"/>
+      <c r="B104" s="50" t="s">
+        <v>86</v>
+      </c>
+      <c r="C104" s="49"/>
       <c r="D104" s="49">
-        <v>65014</v>
+        <v>293189</v>
       </c>
       <c r="E104" s="49">
-        <v>71834</v>
+        <v>201250</v>
       </c>
       <c r="F104" s="49">
-        <v>62464</v>
+        <v>175000</v>
       </c>
       <c r="G104" s="30"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A105" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B105" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="C105" s="33"/>
-      <c r="D105" s="49">
-        <v>103774</v>
-      </c>
-      <c r="E105" s="49">
-        <v>102033</v>
-      </c>
-      <c r="F105" s="49">
-        <v>88724</v>
-      </c>
-      <c r="G105" s="30"/>
+      <c r="A105" s="8"/>
+      <c r="B105" s="9"/>
+      <c r="C105" s="8"/>
+      <c r="D105" s="8"/>
+      <c r="E105" s="8"/>
+      <c r="F105" s="8"/>
+      <c r="G105" s="2"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A106" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B106" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="C106" s="49"/>
-      <c r="D106" s="49">
-        <v>211580</v>
-      </c>
-      <c r="E106" s="49">
-        <v>150513</v>
-      </c>
-      <c r="F106" s="49">
-        <v>130881</v>
-      </c>
-      <c r="G106" s="30"/>
+      <c r="A106" s="8"/>
+      <c r="B106" s="9"/>
+      <c r="C106" s="8"/>
+      <c r="D106" s="8"/>
+      <c r="E106" s="8"/>
+      <c r="F106" s="8"/>
+      <c r="G106" s="2"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A107" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B107" s="50" t="s">
-        <v>85</v>
-      </c>
-      <c r="C107" s="49"/>
-      <c r="D107" s="49">
-        <v>280116</v>
-      </c>
-      <c r="E107" s="49">
-        <v>173234</v>
-      </c>
-      <c r="F107" s="49">
-        <v>150638</v>
-      </c>
-      <c r="G107" s="30"/>
+      <c r="A107" s="8"/>
+      <c r="B107" s="9"/>
+      <c r="C107" s="8"/>
+      <c r="D107" s="8"/>
+      <c r="E107" s="8"/>
+      <c r="F107" s="8"/>
+      <c r="G107" s="2"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A108" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B108" s="50" t="s">
-        <v>79</v>
-      </c>
-      <c r="C108" s="49"/>
-      <c r="D108" s="49">
-        <v>287958</v>
-      </c>
-      <c r="E108" s="49">
-        <v>197111</v>
-      </c>
-      <c r="F108" s="33">
-        <v>171401</v>
-      </c>
-      <c r="G108" s="30"/>
+      <c r="A108" s="8"/>
+      <c r="B108" s="9"/>
+      <c r="C108" s="8"/>
+      <c r="D108" s="8"/>
+      <c r="E108" s="8"/>
+      <c r="F108" s="8"/>
+      <c r="G108" s="2"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A109" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B109" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="C109" s="49"/>
-      <c r="D109" s="49">
-        <v>293189</v>
-      </c>
-      <c r="E109" s="49">
-        <v>201250</v>
-      </c>
-      <c r="F109" s="49">
-        <v>175000</v>
-      </c>
-      <c r="G109" s="30"/>
+      <c r="A109" s="8"/>
+      <c r="B109" s="9"/>
+      <c r="C109" s="8"/>
+      <c r="D109" s="8"/>
+      <c r="E109" s="8"/>
+      <c r="F109" s="8"/>
+      <c r="G109" s="2"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" s="8"/>
@@ -21358,51 +21308,6 @@
       <c r="E997" s="8"/>
       <c r="F997" s="8"/>
       <c r="G997" s="2"/>
-    </row>
-    <row r="998" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A998" s="8"/>
-      <c r="B998" s="9"/>
-      <c r="C998" s="8"/>
-      <c r="D998" s="8"/>
-      <c r="E998" s="8"/>
-      <c r="F998" s="8"/>
-      <c r="G998" s="2"/>
-    </row>
-    <row r="999" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A999" s="8"/>
-      <c r="B999" s="9"/>
-      <c r="C999" s="8"/>
-      <c r="D999" s="8"/>
-      <c r="E999" s="8"/>
-      <c r="F999" s="8"/>
-      <c r="G999" s="2"/>
-    </row>
-    <row r="1000" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1000" s="8"/>
-      <c r="B1000" s="9"/>
-      <c r="C1000" s="8"/>
-      <c r="D1000" s="8"/>
-      <c r="E1000" s="8"/>
-      <c r="F1000" s="8"/>
-      <c r="G1000" s="2"/>
-    </row>
-    <row r="1001" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1001" s="8"/>
-      <c r="B1001" s="9"/>
-      <c r="C1001" s="8"/>
-      <c r="D1001" s="8"/>
-      <c r="E1001" s="8"/>
-      <c r="F1001" s="8"/>
-      <c r="G1001" s="2"/>
-    </row>
-    <row r="1002" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1002" s="8"/>
-      <c r="B1002" s="9"/>
-      <c r="C1002" s="8"/>
-      <c r="D1002" s="8"/>
-      <c r="E1002" s="8"/>
-      <c r="F1002" s="8"/>
-      <c r="G1002" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
data change for cisual cehck
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/MaryCathryn.Lord/Desktop/CoD_PerformanceDash_External/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC532635-3796-C94F-BAEF-8580074E06FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EAF88F9-1BBE-B44B-A068-D2652178AD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="71100" yWindow="-7380" windowWidth="30240" windowHeight="19000" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="511">
   <si>
     <t>KPI tracking workbook</t>
   </si>
@@ -1572,6 +1572,9 @@
   </si>
   <si>
     <t>LIB-CIRCULATION</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -11369,7 +11372,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G997"/>
+  <dimension ref="A1:G1002"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -12865,16 +12868,16 @@
         <v>84</v>
       </c>
       <c r="C82" s="51" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D82" s="49">
-        <v>55</v>
+        <v>143</v>
       </c>
       <c r="E82" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F82" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="G82" s="30"/>
     </row>
@@ -12886,16 +12889,16 @@
         <v>77</v>
       </c>
       <c r="C83" s="51" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D83" s="49">
-        <v>48</v>
+        <v>146</v>
       </c>
       <c r="E83" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F83" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="G83" s="30"/>
     </row>
@@ -12907,16 +12910,16 @@
         <v>85</v>
       </c>
       <c r="C84" s="51" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D84" s="49">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="E84" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F84" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="G84" s="30"/>
     </row>
@@ -12928,16 +12931,16 @@
         <v>79</v>
       </c>
       <c r="C85" s="51" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D85" s="49">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="E85" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F85" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="G85" s="30"/>
     </row>
@@ -12949,16 +12952,16 @@
         <v>86</v>
       </c>
       <c r="C86" s="51" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D86" s="49">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="E86" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F86" s="49">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="G86" s="30"/>
     </row>
@@ -12970,10 +12973,10 @@
         <v>84</v>
       </c>
       <c r="C87" s="51" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D87" s="49">
-        <v>88</v>
+        <v>55</v>
       </c>
       <c r="E87" s="49">
         <v>50</v>
@@ -12991,10 +12994,10 @@
         <v>77</v>
       </c>
       <c r="C88" s="51" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D88" s="49">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="E88" s="49">
         <v>50</v>
@@ -13012,10 +13015,10 @@
         <v>85</v>
       </c>
       <c r="C89" s="51" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D89" s="49">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E89" s="49">
         <v>50</v>
@@ -13033,10 +13036,10 @@
         <v>79</v>
       </c>
       <c r="C90" s="51" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D90" s="49">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="E90" s="49">
         <v>50</v>
@@ -13054,10 +13057,10 @@
         <v>86</v>
       </c>
       <c r="C91" s="51" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D91" s="49">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E91" s="49">
         <v>50</v>
@@ -13069,72 +13072,112 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" s="28" t="s">
-        <v>453</v>
-      </c>
-      <c r="B92" s="49" t="s">
-        <v>489</v>
-      </c>
-      <c r="C92" s="49"/>
-      <c r="D92" s="49"/>
-      <c r="E92" s="49"/>
-      <c r="F92" s="49"/>
+        <v>509</v>
+      </c>
+      <c r="B92" s="50" t="s">
+        <v>84</v>
+      </c>
+      <c r="C92" s="51" t="s">
+        <v>508</v>
+      </c>
+      <c r="D92" s="49">
+        <v>88</v>
+      </c>
+      <c r="E92" s="49">
+        <v>50</v>
+      </c>
+      <c r="F92" s="49">
+        <v>50</v>
+      </c>
       <c r="G92" s="30"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" s="28" t="s">
-        <v>506</v>
-      </c>
-      <c r="B93" s="49" t="s">
-        <v>489</v>
-      </c>
-      <c r="C93" s="49"/>
-      <c r="D93" s="49"/>
-      <c r="E93" s="49"/>
-      <c r="F93" s="49"/>
+        <v>509</v>
+      </c>
+      <c r="B93" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="C93" s="51" t="s">
+        <v>508</v>
+      </c>
+      <c r="D93" s="49">
+        <v>98</v>
+      </c>
+      <c r="E93" s="49">
+        <v>50</v>
+      </c>
+      <c r="F93" s="49">
+        <v>50</v>
+      </c>
       <c r="G93" s="30"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" s="28" t="s">
-        <v>454</v>
-      </c>
-      <c r="B94" s="49" t="s">
-        <v>489</v>
-      </c>
-      <c r="C94" s="49"/>
-      <c r="D94" s="49"/>
-      <c r="E94" s="49"/>
-      <c r="F94" s="49"/>
+        <v>509</v>
+      </c>
+      <c r="B94" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="C94" s="51" t="s">
+        <v>508</v>
+      </c>
+      <c r="D94" s="49">
+        <v>22</v>
+      </c>
+      <c r="E94" s="49">
+        <v>50</v>
+      </c>
+      <c r="F94" s="49">
+        <v>50</v>
+      </c>
       <c r="G94" s="30"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" s="28" t="s">
-        <v>455</v>
-      </c>
-      <c r="B95" s="49" t="s">
-        <v>489</v>
-      </c>
-      <c r="C95" s="49"/>
-      <c r="D95" s="49"/>
-      <c r="E95" s="49"/>
-      <c r="F95" s="49"/>
+        <v>509</v>
+      </c>
+      <c r="B95" s="50" t="s">
+        <v>79</v>
+      </c>
+      <c r="C95" s="51" t="s">
+        <v>508</v>
+      </c>
+      <c r="D95" s="49">
+        <v>54</v>
+      </c>
+      <c r="E95" s="49">
+        <v>50</v>
+      </c>
+      <c r="F95" s="49">
+        <v>50</v>
+      </c>
       <c r="G95" s="30"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" s="28" t="s">
-        <v>456</v>
-      </c>
-      <c r="B96" s="49" t="s">
-        <v>489</v>
-      </c>
-      <c r="C96" s="49"/>
-      <c r="D96" s="49"/>
-      <c r="E96" s="49"/>
-      <c r="F96" s="49"/>
+        <v>509</v>
+      </c>
+      <c r="B96" s="50" t="s">
+        <v>86</v>
+      </c>
+      <c r="C96" s="51" t="s">
+        <v>508</v>
+      </c>
+      <c r="D96" s="49">
+        <v>58</v>
+      </c>
+      <c r="E96" s="49">
+        <v>50</v>
+      </c>
+      <c r="F96" s="49">
+        <v>50</v>
+      </c>
       <c r="G96" s="30"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" s="28" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="B97" s="49" t="s">
         <v>489</v>
@@ -13147,7 +13190,7 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" s="28" t="s">
-        <v>458</v>
+        <v>506</v>
       </c>
       <c r="B98" s="49" t="s">
         <v>489</v>
@@ -13160,162 +13203,182 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" s="28" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B99" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="C99" s="33"/>
-      <c r="D99" s="49">
-        <v>65014</v>
-      </c>
-      <c r="E99" s="49">
-        <v>71834</v>
-      </c>
-      <c r="F99" s="49">
-        <v>62464</v>
-      </c>
+        <v>489</v>
+      </c>
+      <c r="C99" s="49"/>
+      <c r="D99" s="49"/>
+      <c r="E99" s="49"/>
+      <c r="F99" s="49"/>
       <c r="G99" s="30"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B100" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="C100" s="33"/>
-      <c r="D100" s="49">
-        <v>103774</v>
-      </c>
-      <c r="E100" s="49">
-        <v>102033</v>
-      </c>
-      <c r="F100" s="49">
-        <v>88724</v>
-      </c>
+        <v>455</v>
+      </c>
+      <c r="B100" s="49" t="s">
+        <v>489</v>
+      </c>
+      <c r="C100" s="49"/>
+      <c r="D100" s="49"/>
+      <c r="E100" s="49"/>
+      <c r="F100" s="49"/>
       <c r="G100" s="30"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B101" s="50" t="s">
-        <v>77</v>
+        <v>456</v>
+      </c>
+      <c r="B101" s="49" t="s">
+        <v>489</v>
       </c>
       <c r="C101" s="49"/>
-      <c r="D101" s="49">
-        <v>211580</v>
-      </c>
-      <c r="E101" s="49">
-        <v>150513</v>
-      </c>
-      <c r="F101" s="49">
-        <v>130881</v>
-      </c>
+      <c r="D101" s="49"/>
+      <c r="E101" s="49"/>
+      <c r="F101" s="49"/>
       <c r="G101" s="30"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B102" s="50" t="s">
-        <v>85</v>
+        <v>457</v>
+      </c>
+      <c r="B102" s="49" t="s">
+        <v>489</v>
       </c>
       <c r="C102" s="49"/>
-      <c r="D102" s="49">
-        <v>280116</v>
-      </c>
-      <c r="E102" s="49">
-        <v>173234</v>
-      </c>
-      <c r="F102" s="49">
-        <v>150638</v>
-      </c>
+      <c r="D102" s="49"/>
+      <c r="E102" s="49"/>
+      <c r="F102" s="49"/>
       <c r="G102" s="30"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="B103" s="50" t="s">
-        <v>79</v>
+        <v>458</v>
+      </c>
+      <c r="B103" s="49" t="s">
+        <v>489</v>
       </c>
       <c r="C103" s="49"/>
-      <c r="D103" s="49">
-        <v>287958</v>
-      </c>
-      <c r="E103" s="49">
-        <v>197111</v>
-      </c>
-      <c r="F103" s="33">
-        <v>171401</v>
-      </c>
+      <c r="D103" s="49"/>
+      <c r="E103" s="49"/>
+      <c r="F103" s="49"/>
       <c r="G103" s="30"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" s="28" t="s">
         <v>452</v>
       </c>
-      <c r="B104" s="50" t="s">
+      <c r="B104" s="49" t="s">
+        <v>83</v>
+      </c>
+      <c r="C104" s="33"/>
+      <c r="D104" s="49">
+        <v>65014</v>
+      </c>
+      <c r="E104" s="49">
+        <v>71834</v>
+      </c>
+      <c r="F104" s="49">
+        <v>62464</v>
+      </c>
+      <c r="G104" s="30"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A105" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="B105" s="50" t="s">
+        <v>84</v>
+      </c>
+      <c r="C105" s="33"/>
+      <c r="D105" s="49">
+        <v>103774</v>
+      </c>
+      <c r="E105" s="49">
+        <v>102033</v>
+      </c>
+      <c r="F105" s="49">
+        <v>88724</v>
+      </c>
+      <c r="G105" s="30"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="B106" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="C106" s="49"/>
+      <c r="D106" s="49">
+        <v>211580</v>
+      </c>
+      <c r="E106" s="49">
+        <v>150513</v>
+      </c>
+      <c r="F106" s="49">
+        <v>130881</v>
+      </c>
+      <c r="G106" s="30"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A107" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="B107" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="C107" s="49"/>
+      <c r="D107" s="49">
+        <v>280116</v>
+      </c>
+      <c r="E107" s="49">
+        <v>173234</v>
+      </c>
+      <c r="F107" s="49">
+        <v>150638</v>
+      </c>
+      <c r="G107" s="30"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A108" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="B108" s="50" t="s">
+        <v>79</v>
+      </c>
+      <c r="C108" s="49"/>
+      <c r="D108" s="49">
+        <v>287958</v>
+      </c>
+      <c r="E108" s="49">
+        <v>197111</v>
+      </c>
+      <c r="F108" s="33">
+        <v>171401</v>
+      </c>
+      <c r="G108" s="30"/>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="B109" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="C104" s="49"/>
-      <c r="D104" s="49">
+      <c r="C109" s="49"/>
+      <c r="D109" s="49">
         <v>293189</v>
       </c>
-      <c r="E104" s="49">
+      <c r="E109" s="49">
         <v>201250</v>
       </c>
-      <c r="F104" s="49">
+      <c r="F109" s="49">
         <v>175000</v>
       </c>
-      <c r="G104" s="30"/>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A105" s="8"/>
-      <c r="B105" s="9"/>
-      <c r="C105" s="8"/>
-      <c r="D105" s="8"/>
-      <c r="E105" s="8"/>
-      <c r="F105" s="8"/>
-      <c r="G105" s="2"/>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A106" s="8"/>
-      <c r="B106" s="9"/>
-      <c r="C106" s="8"/>
-      <c r="D106" s="8"/>
-      <c r="E106" s="8"/>
-      <c r="F106" s="8"/>
-      <c r="G106" s="2"/>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A107" s="8"/>
-      <c r="B107" s="9"/>
-      <c r="C107" s="8"/>
-      <c r="D107" s="8"/>
-      <c r="E107" s="8"/>
-      <c r="F107" s="8"/>
-      <c r="G107" s="2"/>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A108" s="8"/>
-      <c r="B108" s="9"/>
-      <c r="C108" s="8"/>
-      <c r="D108" s="8"/>
-      <c r="E108" s="8"/>
-      <c r="F108" s="8"/>
-      <c r="G108" s="2"/>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A109" s="8"/>
-      <c r="B109" s="9"/>
-      <c r="C109" s="8"/>
-      <c r="D109" s="8"/>
-      <c r="E109" s="8"/>
-      <c r="F109" s="8"/>
-      <c r="G109" s="2"/>
+      <c r="G109" s="30"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" s="8"/>
@@ -21308,6 +21371,51 @@
       <c r="E997" s="8"/>
       <c r="F997" s="8"/>
       <c r="G997" s="2"/>
+    </row>
+    <row r="998" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A998" s="8"/>
+      <c r="B998" s="9"/>
+      <c r="C998" s="8"/>
+      <c r="D998" s="8"/>
+      <c r="E998" s="8"/>
+      <c r="F998" s="8"/>
+      <c r="G998" s="2"/>
+    </row>
+    <row r="999" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A999" s="8"/>
+      <c r="B999" s="9"/>
+      <c r="C999" s="8"/>
+      <c r="D999" s="8"/>
+      <c r="E999" s="8"/>
+      <c r="F999" s="8"/>
+      <c r="G999" s="2"/>
+    </row>
+    <row r="1000" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1000" s="8"/>
+      <c r="B1000" s="9"/>
+      <c r="C1000" s="8"/>
+      <c r="D1000" s="8"/>
+      <c r="E1000" s="8"/>
+      <c r="F1000" s="8"/>
+      <c r="G1000" s="2"/>
+    </row>
+    <row r="1001" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1001" s="8"/>
+      <c r="B1001" s="9"/>
+      <c r="C1001" s="8"/>
+      <c r="D1001" s="8"/>
+      <c r="E1001" s="8"/>
+      <c r="F1001" s="8"/>
+      <c r="G1001" s="2"/>
+    </row>
+    <row r="1002" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1002" s="8"/>
+      <c r="B1002" s="9"/>
+      <c r="C1002" s="8"/>
+      <c r="D1002" s="8"/>
+      <c r="E1002" s="8"/>
+      <c r="F1002" s="8"/>
+      <c r="G1002" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
adding grant spend and nights on tour data
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -15073,11 +15073,13 @@
         <f>IF(G82="","",IF(ISNUMBER(SEARCH(",",G82)),"Several items (the script lists them)",IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(G82,'Dashboard Items'!$A$2:$A$495,0))&amp;": "&amp;INDEX('Dashboard Items'!$C$2:$C$495,MATCH(G82,'Dashboard Items'!$A$2:$A$495,0)),"ID not found")))</f>
         <v/>
       </c>
-      <c r="I82" s="130" t="s">
-        <v>550</v>
+      <c r="I82" s="130" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
       </c>
       <c r="J82" s="130">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K82" s="130" t="s">
         <v>551</v>
@@ -15100,8 +15102,16 @@
       <c r="Q82" s="130" t="s">
         <v>668</v>
       </c>
-      <c r="R82" s="130"/>
-      <c r="S82" s="130"/>
+      <c r="R82" s="130" t="inlineStr">
+        <is>
+          <t>Submittable grant reimbursement forms (local spend reported), with some manual adjustments</t>
+        </is>
+      </c>
+      <c r="S82" s="130" t="inlineStr">
+        <is>
+          <t>Money spent locally by grant recipients, as reported on their reimbursement forms, for Lodgers' Tax Arts and Culture, Local Event Marketing, Re:New and Durango Creates! grants. Counted by the year of the grant round.</t>
+        </is>
+      </c>
       <c r="T82" s="130"/>
       <c r="U82" s="99" t="str">
         <f>IF(B82="","",IF(IF(D82&lt;&gt;"",D82,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E82,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O82="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D82&lt;&gt;"",D82,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E82,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G82)),IF(O82="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O82="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D82&lt;&gt;"",D82,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E82,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
@@ -15140,7 +15150,7 @@
         <v>550</v>
       </c>
       <c r="J83" s="130">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K83" s="130" t="s">
         <v>551</v>
@@ -15164,8 +15174,16 @@
         <v>668</v>
       </c>
       <c r="R83" s="130"/>
-      <c r="S83" s="130"/>
-      <c r="T83" s="130"/>
+      <c r="S83" s="130" t="inlineStr">
+        <is>
+          <t>Room nights sold during the year to new tour companies, meeting planners and FIT (independent traveler) contracts, including nights booked now for stays in later years.</t>
+        </is>
+      </c>
+      <c r="T83" s="130" t="inlineStr">
+        <is>
+          <t>Counts new organizations only. Ongoing accounts are not included; for example, the two Tauck Tours series sold in 2024 bring about 400 room nights a year but are not in the 2026 count.</t>
+        </is>
+      </c>
       <c r="U83" s="99" t="str">
         <f>IF(B83="","",IF(IF(D83&lt;&gt;"",D83,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E83,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O83="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D83&lt;&gt;"",D83,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E83,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G83)),IF(O83="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O83="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D83&lt;&gt;"",D83,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E83,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
         <v>Sets Program status chip</v>
@@ -25957,7 +25975,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="138" spans="1:7" s="130" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:8" s="130" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="130" t="str">
         <f t="shared" si="2"/>
         <v>PROS</v>
@@ -25965,8 +25983,21 @@
       <c r="B138" s="130" t="s">
         <v>671</v>
       </c>
+      <c r="C138" s="130" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E138" s="130">
+        <v>121350.25</v>
+      </c>
       <c r="F138" s="130">
         <v>368438</v>
+      </c>
+      <c r="H138" s="130" t="inlineStr">
+        <is>
+          <t>Year to date as of Oct 15, 2026; 2026 grant reimbursements are still coming in</t>
+        </is>
       </c>
     </row>
     <row r="139" spans="1:7" s="130" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26003,7 +26034,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:7" s="130" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:8" s="130" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="130" t="str">
         <f t="shared" si="2"/>
         <v>PROS</v>
@@ -26011,8 +26042,21 @@
       <c r="B142" s="130" t="s">
         <v>672</v>
       </c>
+      <c r="C142" s="130" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E142" s="130">
+        <v>1949</v>
+      </c>
       <c r="F142" s="130">
         <v>1000</v>
+      </c>
+      <c r="H142" s="130" t="inlineStr">
+        <is>
+          <t>Estimate as of Oct 21, 2026: nights already stayed plus nights booked for later stays (e.g., Model A Ford Club, June 2027)</t>
+        </is>
       </c>
     </row>
     <row r="143" spans="1:7" s="130" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -28751,10 +28795,24 @@
       <c r="H293" s="161"/>
     </row>
     <row r="294" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B294" s="163"/>
-      <c r="C294" s="159"/>
+      <c r="A294" s="130" t="str">
+        <f>LEFT(B294, FIND("-", B294) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B294" s="130" t="inlineStr">
+        <is>
+          <t>PROS-LOCALSPEND</t>
+        </is>
+      </c>
+      <c r="C294" s="159" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="D294" s="160"/>
-      <c r="E294" s="160"/>
+      <c r="E294" s="160">
+        <v>342859.57</v>
+      </c>
       <c r="F294" s="160"/>
       <c r="G294" s="160"/>
       <c r="H294" s="161"/>

</xml_diff>

<commit_message>
moving housing out of bjective 6.3
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -39560,27 +39560,23 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="149" t="s">
-        <v>681</v>
-      </c>
+      <c r="A27" s="149"/>
       <c r="B27" s="85" t="str">
         <f>IF(A27="","",IFERROR(INDEX('Dashboard Items'!$C$2:$C$495,MATCH(A27,'Dashboard Items'!$A$2:$A$495,0)),"ID not found"))</f>
-        <v>Community Development &amp; Planning</v>
+        <v/>
       </c>
       <c r="C27" s="85" t="str">
         <f>IF(A27="","",IFERROR(INDEX('Dashboard Items'!$E$2:$E$495,MATCH(A27,'Dashboard Items'!$A$2:$A$495,0)),"ID not found"))</f>
-        <v>Community Growth and Economic Vitality</v>
-      </c>
-      <c r="D27" s="149" t="s">
-        <v>931</v>
-      </c>
+        <v/>
+      </c>
+      <c r="D27" s="149"/>
       <c r="E27" s="85" t="str">
         <f>IF(D27="","",IFERROR(INDEX('Dashboard Items'!$C$2:$C$495,MATCH(D27,'Dashboard Items'!$A$2:$A$495,0)),"ID not found"))</f>
-        <v>6.1 Employee Growth and Retention</v>
+        <v/>
       </c>
       <c r="F27" s="85" t="str">
         <f>IF(D27="","",IFERROR(INDEX('Dashboard Items'!$F$2:$F$495,MATCH(D27,'Dashboard Items'!$A$2:$A$495,0)),"ID not found"))</f>
-        <v>Strategic Workforce Development</v>
+        <v/>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
pulling data from current dash
</commit_message>
<xml_diff>
--- a/KPI_Tracking.xlsx
+++ b/KPI_Tracking.xlsx
@@ -11431,18 +11431,44 @@
         <f>IF(G9="","",IF(ISNUMBER(SEARCH(",",G9)),"Several items (the script lists them)",IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(G9,'Dashboard Items'!$A$2:$A$495,0))&amp;": "&amp;INDEX('Dashboard Items'!$C$2:$C$495,MATCH(G9,'Dashboard Items'!$A$2:$A$495,0)),"ID not found")))</f>
         <v>Key Service: City Clerk &amp; Records Management</v>
       </c>
-      <c r="I9" s="87"/>
-      <c r="J9" s="87"/>
-      <c r="K9" s="87"/>
-      <c r="L9" s="87"/>
+      <c r="I9" s="87" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="J9" s="87">
+        <v>0</v>
+      </c>
+      <c r="K9" s="87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L9" s="87" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
       <c r="M9" s="87"/>
       <c r="N9" s="87"/>
       <c r="O9" s="87"/>
-      <c r="P9" s="87"/>
+      <c r="P9" s="87" t="inlineStr">
+        <is>
+          <t>Every Quarter</t>
+        </is>
+      </c>
       <c r="Q9" s="87"/>
       <c r="R9" s="87"/>
-      <c r="S9" s="87"/>
-      <c r="T9" s="87"/>
+      <c r="S9" s="87" t="inlineStr">
+        <is>
+          <t>Share of regular City Council meeting agendas posted at least 48 hours before the meeting, each quarter.</t>
+        </is>
+      </c>
+      <c r="T9" s="87" t="inlineStr">
+        <is>
+          <t>Target: more than 90% posted within 48 hours. Results swing from quarter to quarter because the number of meetings varies.</t>
+        </is>
+      </c>
       <c r="U9" s="85" t="str">
         <f>IF(B9="","",IF(IF(D9&lt;&gt;"",D9,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E9,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O9="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D9&lt;&gt;"",D9,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E9,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G9)),IF(O9="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O9="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D9&lt;&gt;"",D9,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E9,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
         <v>Counts in Key Service gauge + sets Program chip</v>
@@ -11564,18 +11590,44 @@
         <f>IF(G12="","",IF(ISNUMBER(SEARCH(",",G12)),"Several items (the script lists them)",IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(G12,'Dashboard Items'!$A$2:$A$495,0))&amp;": "&amp;INDEX('Dashboard Items'!$C$2:$C$495,MATCH(G12,'Dashboard Items'!$A$2:$A$495,0)),"ID not found")))</f>
         <v>Key Service: City Clerk &amp; Records Management</v>
       </c>
-      <c r="I12" s="87"/>
-      <c r="J12" s="87"/>
-      <c r="K12" s="87"/>
-      <c r="L12" s="87"/>
+      <c r="I12" s="87" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="J12" s="87">
+        <v>0</v>
+      </c>
+      <c r="K12" s="87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L12" s="87" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
       <c r="M12" s="87"/>
       <c r="N12" s="87"/>
       <c r="O12" s="87"/>
-      <c r="P12" s="87"/>
+      <c r="P12" s="87" t="inlineStr">
+        <is>
+          <t>Every Quarter</t>
+        </is>
+      </c>
       <c r="Q12" s="87"/>
       <c r="R12" s="87"/>
-      <c r="S12" s="87"/>
-      <c r="T12" s="87"/>
+      <c r="S12" s="87" t="inlineStr">
+        <is>
+          <t>Share of public records requests closed within 24 hours, each quarter.</t>
+        </is>
+      </c>
+      <c r="T12" s="87" t="inlineStr">
+        <is>
+          <t>Target: 90% closed within 24 hours. The legal deadline is 3 days. Some requests are delayed while waiting on the requester, especially for payment.</t>
+        </is>
+      </c>
       <c r="U12" s="85" t="str">
         <f>IF(B12="","",IF(IF(D12&lt;&gt;"",D12,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E12,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O12="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D12&lt;&gt;"",D12,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E12,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G12)),IF(O12="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O12="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D12&lt;&gt;"",D12,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E12,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
         <v>Counts in Key Service gauge + sets Program chip</v>
@@ -12157,18 +12209,44 @@
         <f>IF(G25="","",IF(ISNUMBER(SEARCH(",",G25)),"Several items (the script lists them)",IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(G25,'Dashboard Items'!$A$2:$A$495,0))&amp;": "&amp;INDEX('Dashboard Items'!$C$2:$C$495,MATCH(G25,'Dashboard Items'!$A$2:$A$495,0)),"ID not found")))</f>
         <v>Program: Recruitment &amp; Retention</v>
       </c>
-      <c r="I25" s="81"/>
-      <c r="J25" s="81"/>
-      <c r="K25" s="81"/>
-      <c r="L25" s="81"/>
+      <c r="I25" s="81" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="J25" s="81">
+        <v>2</v>
+      </c>
+      <c r="K25" s="81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L25" s="81" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
       <c r="M25" s="81"/>
       <c r="N25" s="81"/>
       <c r="O25" s="81"/>
-      <c r="P25" s="81"/>
+      <c r="P25" s="81" t="inlineStr">
+        <is>
+          <t>Every year</t>
+        </is>
+      </c>
       <c r="Q25" s="81"/>
       <c r="R25" s="81"/>
-      <c r="S25" s="81"/>
-      <c r="T25" s="81"/>
+      <c r="S25" s="81" t="inlineStr">
+        <is>
+          <t>Internal promotion rate for full-time City positions each fiscal year.</t>
+        </is>
+      </c>
+      <c r="T25" s="81" t="inlineStr">
+        <is>
+          <t>Target: 10%. Benchmark: 6%, SHRM's average internal promotion rate.</t>
+        </is>
+      </c>
       <c r="U25" s="85" t="str">
         <f>IF(B25="","",IF(IF(D25&lt;&gt;"",D25,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E25,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O25="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D25&lt;&gt;"",D25,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E25,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G25)),IF(O25="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O25="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D25&lt;&gt;"",D25,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E25,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
         <v>Counts in Key Service gauge</v>
@@ -12646,18 +12724,44 @@
         <f>IF(G36="","",IF(ISNUMBER(SEARCH(",",G36)),"Several items (the script lists them)",IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(G36,'Dashboard Items'!$A$2:$A$495,0))&amp;": "&amp;INDEX('Dashboard Items'!$C$2:$C$495,MATCH(G36,'Dashboard Items'!$A$2:$A$495,0)),"ID not found")))</f>
         <v>Program: Recruitment &amp; Retention</v>
       </c>
-      <c r="I36" s="81"/>
-      <c r="J36" s="81"/>
-      <c r="K36" s="81"/>
-      <c r="L36" s="81"/>
+      <c r="I36" s="81" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="J36" s="81">
+        <v>2</v>
+      </c>
+      <c r="K36" s="81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" s="81" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
       <c r="M36" s="81"/>
       <c r="N36" s="81"/>
       <c r="O36" s="81"/>
-      <c r="P36" s="81"/>
+      <c r="P36" s="81" t="inlineStr">
+        <is>
+          <t>Every year</t>
+        </is>
+      </c>
       <c r="Q36" s="81"/>
       <c r="R36" s="81"/>
-      <c r="S36" s="81"/>
-      <c r="T36" s="81"/>
+      <c r="S36" s="81" t="inlineStr">
+        <is>
+          <t>Cumulative turnover rate for City employees each fiscal year. Lower is better.</t>
+        </is>
+      </c>
+      <c r="T36" s="81" t="inlineStr">
+        <is>
+          <t>Target: 20%. Benchmark: the Colorado average (18% in 2021, 20% in 2022, 18% in 2023); from 2024, SHRM's 20% average for government, as the Colorado figure is not available. Shown as one total; a voluntary/involuntary split is not available yet.</t>
+        </is>
+      </c>
       <c r="U36" s="85" t="str">
         <f>IF(B36="","",IF(IF(D36&lt;&gt;"",D36,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E36,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O36="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D36&lt;&gt;"",D36,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E36,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G36)),IF(O36="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O36="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D36&lt;&gt;"",D36,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E36,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
         <v>Counts in Key Service gauge</v>
@@ -15244,7 +15348,7 @@
         <v>550</v>
       </c>
       <c r="J79" s="116">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K79" s="116" t="s">
         <v>551</v>
@@ -15268,8 +15372,16 @@
         <v>668</v>
       </c>
       <c r="R79" s="116"/>
-      <c r="S79" s="116"/>
-      <c r="T79" s="116"/>
+      <c r="S79" s="116" t="inlineStr">
+        <is>
+          <t>Community events supported with City services such as production, facilities and equipment, each fiscal year.</t>
+        </is>
+      </c>
+      <c r="T79" s="116" t="inlineStr">
+        <is>
+          <t>Target: 250 events, set from Customer Service portal and self-service capacity. Growth is limited by the calendar and the number of facilities available.</t>
+        </is>
+      </c>
       <c r="U79" s="85" t="str">
         <f>IF(B79="","",IF(IF(D79&lt;&gt;"",D79,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E79,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O79="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D79&lt;&gt;"",D79,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E79,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G79)),IF(O79="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O79="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D79&lt;&gt;"",D79,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E79,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
         <v>Counts in Key Service gauge</v>
@@ -15622,7 +15734,7 @@
         <v>550</v>
       </c>
       <c r="J85" s="116">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K85" s="116" t="s">
         <v>551</v>
@@ -15646,8 +15758,16 @@
         <v>668</v>
       </c>
       <c r="R85" s="116"/>
-      <c r="S85" s="116"/>
-      <c r="T85" s="116"/>
+      <c r="S85" s="116" t="inlineStr">
+        <is>
+          <t>Community event permits issued each fiscal year.</t>
+        </is>
+      </c>
+      <c r="T85" s="116" t="inlineStr">
+        <is>
+          <t>Target: 240 permits, set from Customer Service portal and self-service capacity. Growth is limited by the calendar and the number of facilities available. Counts community event permits only; activity, park and banner permits are not included yet.</t>
+        </is>
+      </c>
       <c r="U85" s="85" t="str">
         <f>IF(B85="","",IF(IF(D85&lt;&gt;"",D85,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E85,'Dashboard Items'!$A$2:$A$495,0)),""))="Key Service",IF(O85="No","Key Service: shown, not counted","Counts in Key Service gauge"),IF(IF(D85&lt;&gt;"",D85,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E85,'Dashboard Items'!$A$2:$A$495,0)),""))="Program",IF(ISNUMBER(SEARCH("ks",G85)),IF(O85="No","Program, also at Key Service: not counted","Counts in Key Service gauge + sets Program chip"),IF(O85="No","Program: shown, no status chip","Sets Program status chip")),IF(IF(D85&lt;&gt;"",D85,IFERROR(INDEX('Dashboard Items'!$B$2:$B$495,MATCH(E85,'Dashboard Items'!$A$2:$A$495,0)),""))="Work System","Work System: shown, not counted","Check Level"))))</f>
         <v>Sets Program status chip</v>
@@ -23696,13 +23816,20 @@
       <c r="B6" s="127" t="s">
         <v>569</v>
       </c>
-      <c r="C6" s="128" t="s">
-        <v>777</v>
+      <c r="C6" s="128" t="inlineStr">
+        <is>
+          <t>2024-Q4</t>
+        </is>
       </c>
       <c r="D6" s="128"/>
-      <c r="E6" s="128"/>
-      <c r="F6" s="128"/>
+      <c r="E6" s="128">
+        <v>88</v>
+      </c>
+      <c r="F6" s="128">
+        <v>90</v>
+      </c>
       <c r="G6" s="128"/>
+      <c r="H6" s="128"/>
     </row>
     <row r="7" spans="1:8" s="127" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="127" t="str">
@@ -23712,13 +23839,20 @@
       <c r="B7" s="127" t="s">
         <v>565</v>
       </c>
-      <c r="C7" s="128" t="s">
-        <v>777</v>
+      <c r="C7" s="128" t="inlineStr">
+        <is>
+          <t>2024-Q4</t>
+        </is>
       </c>
       <c r="D7" s="128"/>
-      <c r="E7" s="128"/>
-      <c r="F7" s="128"/>
+      <c r="E7" s="128">
+        <v>95</v>
+      </c>
+      <c r="F7" s="128">
+        <v>90</v>
+      </c>
       <c r="G7" s="128"/>
+      <c r="H7" s="128"/>
     </row>
     <row r="8" spans="1:8" s="127" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="127" t="str">
@@ -23886,7 +24020,7 @@
       <c r="F16" s="129"/>
       <c r="G16" s="129"/>
     </row>
-    <row r="17" spans="1:7" s="94" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" s="94" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="94" t="str">
         <f t="shared" si="0"/>
         <v>HR</v>
@@ -23894,11 +24028,22 @@
       <c r="B17" s="94" t="s">
         <v>605</v>
       </c>
-      <c r="C17" s="129"/>
+      <c r="C17" s="129" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="D17" s="129"/>
-      <c r="E17" s="129"/>
-      <c r="F17" s="129"/>
-      <c r="G17" s="129"/>
+      <c r="E17" s="129">
+        <v>20.34</v>
+      </c>
+      <c r="F17" s="129">
+        <v>20</v>
+      </c>
+      <c r="G17" s="129">
+        <v>18</v>
+      </c>
+      <c r="H17" s="129"/>
     </row>
     <row r="18" spans="1:7" s="94" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="94" t="str">
@@ -24026,7 +24171,7 @@
       <c r="F26" s="129"/>
       <c r="G26" s="129"/>
     </row>
-    <row r="27" spans="1:7" s="94" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" s="94" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="94" t="str">
         <f t="shared" si="0"/>
         <v>HR</v>
@@ -24034,11 +24179,22 @@
       <c r="B27" s="94" t="s">
         <v>593</v>
       </c>
-      <c r="C27" s="129"/>
+      <c r="C27" s="129" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="D27" s="129"/>
-      <c r="E27" s="129"/>
-      <c r="F27" s="129"/>
-      <c r="G27" s="129"/>
+      <c r="E27" s="129">
+        <v>49.3</v>
+      </c>
+      <c r="F27" s="129">
+        <v>10</v>
+      </c>
+      <c r="G27" s="129">
+        <v>6</v>
+      </c>
+      <c r="H27" s="129"/>
     </row>
     <row r="28" spans="1:7" s="94" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="94" t="str">
@@ -29985,246 +30141,692 @@
       </c>
       <c r="H321" s="147"/>
     </row>
-    <row r="322" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B322" s="149"/>
-      <c r="C322" s="145"/>
+    <row r="322" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A322" s="116" t="str">
+        <f>LEFT(B322, FIND("-", B322) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B322" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-AGENDAPOST</t>
+        </is>
+      </c>
+      <c r="C322" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
       <c r="D322" s="146"/>
-      <c r="E322" s="146"/>
-      <c r="F322" s="146"/>
+      <c r="E322" s="146">
+        <v>95</v>
+      </c>
+      <c r="F322" s="146">
+        <v>90</v>
+      </c>
       <c r="G322" s="146"/>
       <c r="H322" s="147"/>
     </row>
-    <row r="323" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B323" s="149"/>
-      <c r="C323" s="145"/>
+    <row r="323" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A323" s="116" t="str">
+        <f>LEFT(B323, FIND("-", B323) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B323" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-AGENDAPOST</t>
+        </is>
+      </c>
+      <c r="C323" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
       <c r="D323" s="146"/>
-      <c r="E323" s="146"/>
-      <c r="F323" s="146"/>
+      <c r="E323" s="146">
+        <v>95</v>
+      </c>
+      <c r="F323" s="146">
+        <v>90</v>
+      </c>
       <c r="G323" s="146"/>
       <c r="H323" s="147"/>
     </row>
-    <row r="324" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B324" s="149"/>
-      <c r="C324" s="145"/>
+    <row r="324" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A324" s="116" t="str">
+        <f>LEFT(B324, FIND("-", B324) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B324" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-AGENDAPOST</t>
+        </is>
+      </c>
+      <c r="C324" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q3</t>
+        </is>
+      </c>
       <c r="D324" s="146"/>
-      <c r="E324" s="146"/>
-      <c r="F324" s="146"/>
+      <c r="E324" s="146">
+        <v>97</v>
+      </c>
+      <c r="F324" s="146">
+        <v>90</v>
+      </c>
       <c r="G324" s="146"/>
       <c r="H324" s="147"/>
     </row>
-    <row r="325" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B325" s="149"/>
-      <c r="C325" s="145"/>
+    <row r="325" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A325" s="116" t="str">
+        <f>LEFT(B325, FIND("-", B325) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B325" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-AGENDAPOST</t>
+        </is>
+      </c>
+      <c r="C325" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q4</t>
+        </is>
+      </c>
       <c r="D325" s="146"/>
-      <c r="E325" s="146"/>
-      <c r="F325" s="146"/>
+      <c r="E325" s="146">
+        <v>97</v>
+      </c>
+      <c r="F325" s="146">
+        <v>90</v>
+      </c>
       <c r="G325" s="146"/>
       <c r="H325" s="147"/>
     </row>
-    <row r="326" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B326" s="149"/>
-      <c r="C326" s="145"/>
+    <row r="326" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A326" s="116" t="str">
+        <f>LEFT(B326, FIND("-", B326) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B326" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-AGENDAPOST</t>
+        </is>
+      </c>
+      <c r="C326" s="145" t="inlineStr">
+        <is>
+          <t>2026-Q1</t>
+        </is>
+      </c>
       <c r="D326" s="146"/>
-      <c r="E326" s="146"/>
-      <c r="F326" s="146"/>
+      <c r="E326" s="146">
+        <v>95</v>
+      </c>
+      <c r="F326" s="146">
+        <v>90</v>
+      </c>
       <c r="G326" s="146"/>
       <c r="H326" s="147"/>
     </row>
-    <row r="327" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B327" s="149"/>
-      <c r="C327" s="145"/>
+    <row r="327" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A327" s="116" t="str">
+        <f>LEFT(B327, FIND("-", B327) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B327" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-CORARESPRATE</t>
+        </is>
+      </c>
+      <c r="C327" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
       <c r="D327" s="146"/>
-      <c r="E327" s="146"/>
-      <c r="F327" s="146"/>
+      <c r="E327" s="146">
+        <v>87</v>
+      </c>
+      <c r="F327" s="146">
+        <v>90</v>
+      </c>
       <c r="G327" s="146"/>
       <c r="H327" s="147"/>
     </row>
-    <row r="328" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B328" s="149"/>
-      <c r="C328" s="145"/>
+    <row r="328" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A328" s="116" t="str">
+        <f>LEFT(B328, FIND("-", B328) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B328" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-CORARESPRATE</t>
+        </is>
+      </c>
+      <c r="C328" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
       <c r="D328" s="146"/>
-      <c r="E328" s="146"/>
-      <c r="F328" s="146"/>
+      <c r="E328" s="146">
+        <v>87</v>
+      </c>
+      <c r="F328" s="146">
+        <v>90</v>
+      </c>
       <c r="G328" s="146"/>
       <c r="H328" s="147"/>
     </row>
-    <row r="329" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B329" s="149"/>
-      <c r="C329" s="145"/>
+    <row r="329" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A329" s="116" t="str">
+        <f>LEFT(B329, FIND("-", B329) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B329" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-CORARESPRATE</t>
+        </is>
+      </c>
+      <c r="C329" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q3</t>
+        </is>
+      </c>
       <c r="D329" s="146"/>
-      <c r="E329" s="146"/>
-      <c r="F329" s="146"/>
+      <c r="E329" s="146">
+        <v>88</v>
+      </c>
+      <c r="F329" s="146">
+        <v>90</v>
+      </c>
       <c r="G329" s="146"/>
       <c r="H329" s="147"/>
     </row>
-    <row r="330" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B330" s="149"/>
-      <c r="C330" s="145"/>
+    <row r="330" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A330" s="116" t="str">
+        <f>LEFT(B330, FIND("-", B330) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B330" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-CORARESPRATE</t>
+        </is>
+      </c>
+      <c r="C330" s="145" t="inlineStr">
+        <is>
+          <t>2025-Q4</t>
+        </is>
+      </c>
       <c r="D330" s="146"/>
-      <c r="E330" s="146"/>
-      <c r="F330" s="146"/>
+      <c r="E330" s="146">
+        <v>88</v>
+      </c>
+      <c r="F330" s="146">
+        <v>90</v>
+      </c>
       <c r="G330" s="146"/>
       <c r="H330" s="147"/>
     </row>
-    <row r="331" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B331" s="149"/>
-      <c r="C331" s="145"/>
+    <row r="331" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A331" s="116" t="str">
+        <f>LEFT(B331, FIND("-", B331) - 1)</f>
+        <v>CLERK</v>
+      </c>
+      <c r="B331" s="116" t="inlineStr">
+        <is>
+          <t>CLERK-CORARESPRATE</t>
+        </is>
+      </c>
+      <c r="C331" s="145" t="inlineStr">
+        <is>
+          <t>2026-Q1</t>
+        </is>
+      </c>
       <c r="D331" s="146"/>
-      <c r="E331" s="146"/>
-      <c r="F331" s="146"/>
+      <c r="E331" s="146">
+        <v>88</v>
+      </c>
+      <c r="F331" s="146">
+        <v>90</v>
+      </c>
       <c r="G331" s="146"/>
       <c r="H331" s="147"/>
     </row>
-    <row r="332" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B332" s="149"/>
-      <c r="C332" s="145"/>
+    <row r="332" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A332" s="116" t="str">
+        <f>LEFT(B332, FIND("-", B332) - 1)</f>
+        <v>HR</v>
+      </c>
+      <c r="B332" s="116" t="inlineStr">
+        <is>
+          <t>HR-TURNRATE</t>
+        </is>
+      </c>
+      <c r="C332" s="145" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="D332" s="146"/>
-      <c r="E332" s="146"/>
-      <c r="F332" s="146"/>
-      <c r="G332" s="146"/>
+      <c r="E332" s="146">
+        <v>20.3</v>
+      </c>
+      <c r="F332" s="146">
+        <v>20</v>
+      </c>
+      <c r="G332" s="146">
+        <v>20</v>
+      </c>
       <c r="H332" s="147"/>
     </row>
-    <row r="333" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B333" s="149"/>
-      <c r="C333" s="145"/>
+    <row r="333" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A333" s="116" t="str">
+        <f>LEFT(B333, FIND("-", B333) - 1)</f>
+        <v>HR</v>
+      </c>
+      <c r="B333" s="116" t="inlineStr">
+        <is>
+          <t>HR-TURNRATE</t>
+        </is>
+      </c>
+      <c r="C333" s="145" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="D333" s="146"/>
-      <c r="E333" s="146"/>
-      <c r="F333" s="146"/>
-      <c r="G333" s="146"/>
+      <c r="E333" s="146">
+        <v>21.18</v>
+      </c>
+      <c r="F333" s="146">
+        <v>20</v>
+      </c>
+      <c r="G333" s="146">
+        <v>18</v>
+      </c>
       <c r="H333" s="147"/>
     </row>
-    <row r="334" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B334" s="149"/>
-      <c r="C334" s="145"/>
+    <row r="334" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A334" s="116" t="str">
+        <f>LEFT(B334, FIND("-", B334) - 1)</f>
+        <v>HR</v>
+      </c>
+      <c r="B334" s="116" t="inlineStr">
+        <is>
+          <t>HR-TURNRATE</t>
+        </is>
+      </c>
+      <c r="C334" s="145" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="D334" s="146"/>
-      <c r="E334" s="146"/>
-      <c r="F334" s="146"/>
-      <c r="G334" s="146"/>
+      <c r="E334" s="146">
+        <v>19.85</v>
+      </c>
+      <c r="F334" s="146">
+        <v>20</v>
+      </c>
+      <c r="G334" s="146">
+        <v>20</v>
+      </c>
       <c r="H334" s="147"/>
     </row>
-    <row r="335" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B335" s="149"/>
-      <c r="C335" s="145"/>
+    <row r="335" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A335" s="116" t="str">
+        <f>LEFT(B335, FIND("-", B335) - 1)</f>
+        <v>HR</v>
+      </c>
+      <c r="B335" s="116" t="inlineStr">
+        <is>
+          <t>HR-TURNRATE</t>
+        </is>
+      </c>
+      <c r="C335" s="145" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="D335" s="146"/>
-      <c r="E335" s="146"/>
-      <c r="F335" s="146"/>
-      <c r="G335" s="146"/>
+      <c r="E335" s="146">
+        <v>16.6</v>
+      </c>
+      <c r="F335" s="146">
+        <v>20</v>
+      </c>
+      <c r="G335" s="146">
+        <v>20</v>
+      </c>
       <c r="H335" s="147"/>
     </row>
-    <row r="336" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B336" s="149"/>
-      <c r="C336" s="145"/>
+    <row r="336" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A336" s="116" t="str">
+        <f>LEFT(B336, FIND("-", B336) - 1)</f>
+        <v>HR</v>
+      </c>
+      <c r="B336" s="116" t="inlineStr">
+        <is>
+          <t>HR-INTPROMO</t>
+        </is>
+      </c>
+      <c r="C336" s="145" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="D336" s="146"/>
-      <c r="E336" s="146"/>
-      <c r="F336" s="146"/>
-      <c r="G336" s="146"/>
+      <c r="E336" s="146">
+        <v>20.6</v>
+      </c>
+      <c r="F336" s="146">
+        <v>10</v>
+      </c>
+      <c r="G336" s="146">
+        <v>6</v>
+      </c>
       <c r="H336" s="147"/>
     </row>
-    <row r="337" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B337" s="149"/>
-      <c r="C337" s="145"/>
+    <row r="337" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A337" s="116" t="str">
+        <f>LEFT(B337, FIND("-", B337) - 1)</f>
+        <v>HR</v>
+      </c>
+      <c r="B337" s="116" t="inlineStr">
+        <is>
+          <t>HR-INTPROMO</t>
+        </is>
+      </c>
+      <c r="C337" s="145" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="D337" s="146"/>
-      <c r="E337" s="146"/>
-      <c r="F337" s="146"/>
-      <c r="G337" s="146"/>
+      <c r="E337" s="146">
+        <v>17.6</v>
+      </c>
+      <c r="F337" s="146">
+        <v>10</v>
+      </c>
+      <c r="G337" s="146">
+        <v>6</v>
+      </c>
       <c r="H337" s="147"/>
     </row>
-    <row r="338" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B338" s="149"/>
-      <c r="C338" s="145"/>
+    <row r="338" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A338" s="116" t="str">
+        <f>LEFT(B338, FIND("-", B338) - 1)</f>
+        <v>HR</v>
+      </c>
+      <c r="B338" s="116" t="inlineStr">
+        <is>
+          <t>HR-INTPROMO</t>
+        </is>
+      </c>
+      <c r="C338" s="145" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="D338" s="146"/>
-      <c r="E338" s="146"/>
-      <c r="F338" s="146"/>
-      <c r="G338" s="146"/>
+      <c r="E338" s="146">
+        <v>30.09</v>
+      </c>
+      <c r="F338" s="146">
+        <v>10</v>
+      </c>
+      <c r="G338" s="146">
+        <v>6</v>
+      </c>
       <c r="H338" s="147"/>
     </row>
-    <row r="339" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B339" s="149"/>
-      <c r="C339" s="145"/>
+    <row r="339" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A339" s="116" t="str">
+        <f>LEFT(B339, FIND("-", B339) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B339" s="116" t="inlineStr">
+        <is>
+          <t>PROS-ALLCOMMEVENTS</t>
+        </is>
+      </c>
+      <c r="C339" s="145" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
       <c r="D339" s="146"/>
-      <c r="E339" s="146"/>
-      <c r="F339" s="146"/>
+      <c r="E339" s="146">
+        <v>47</v>
+      </c>
+      <c r="F339" s="146">
+        <v>250</v>
+      </c>
       <c r="G339" s="146"/>
       <c r="H339" s="147"/>
     </row>
-    <row r="340" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B340" s="149"/>
-      <c r="C340" s="145"/>
+    <row r="340" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A340" s="116" t="str">
+        <f>LEFT(B340, FIND("-", B340) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B340" s="116" t="inlineStr">
+        <is>
+          <t>PROS-ALLCOMMEVENTS</t>
+        </is>
+      </c>
+      <c r="C340" s="145" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="D340" s="146"/>
-      <c r="E340" s="146"/>
-      <c r="F340" s="146"/>
+      <c r="E340" s="146">
+        <v>202</v>
+      </c>
+      <c r="F340" s="146">
+        <v>250</v>
+      </c>
       <c r="G340" s="146"/>
       <c r="H340" s="147"/>
     </row>
-    <row r="341" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B341" s="149"/>
-      <c r="C341" s="145"/>
+    <row r="341" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A341" s="116" t="str">
+        <f>LEFT(B341, FIND("-", B341) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B341" s="116" t="inlineStr">
+        <is>
+          <t>PROS-ALLCOMMEVENTS</t>
+        </is>
+      </c>
+      <c r="C341" s="145" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="D341" s="146"/>
-      <c r="E341" s="146"/>
-      <c r="F341" s="146"/>
+      <c r="E341" s="146">
+        <v>264</v>
+      </c>
+      <c r="F341" s="146">
+        <v>250</v>
+      </c>
       <c r="G341" s="146"/>
       <c r="H341" s="147"/>
     </row>
-    <row r="342" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B342" s="149"/>
-      <c r="C342" s="145"/>
+    <row r="342" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A342" s="116" t="str">
+        <f>LEFT(B342, FIND("-", B342) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B342" s="116" t="inlineStr">
+        <is>
+          <t>PROS-ALLCOMMEVENTS</t>
+        </is>
+      </c>
+      <c r="C342" s="145" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="D342" s="146"/>
-      <c r="E342" s="146"/>
-      <c r="F342" s="146"/>
+      <c r="E342" s="146">
+        <v>236</v>
+      </c>
+      <c r="F342" s="146">
+        <v>250</v>
+      </c>
       <c r="G342" s="146"/>
       <c r="H342" s="147"/>
     </row>
-    <row r="343" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B343" s="149"/>
-      <c r="C343" s="145"/>
+    <row r="343" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A343" s="116" t="str">
+        <f>LEFT(B343, FIND("-", B343) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B343" s="116" t="inlineStr">
+        <is>
+          <t>PROS-ALLCOMMEVENTS</t>
+        </is>
+      </c>
+      <c r="C343" s="145" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="D343" s="146"/>
-      <c r="E343" s="146"/>
-      <c r="F343" s="146"/>
+      <c r="E343" s="146">
+        <v>236</v>
+      </c>
+      <c r="F343" s="146">
+        <v>250</v>
+      </c>
       <c r="G343" s="146"/>
       <c r="H343" s="147"/>
     </row>
-    <row r="344" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B344" s="149"/>
-      <c r="C344" s="145"/>
+    <row r="344" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A344" s="116" t="str">
+        <f>LEFT(B344, FIND("-", B344) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B344" s="116" t="inlineStr">
+        <is>
+          <t>PROS-ALLCOMMEVENTS</t>
+        </is>
+      </c>
+      <c r="C344" s="145" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="D344" s="146"/>
-      <c r="E344" s="146"/>
-      <c r="F344" s="146"/>
+      <c r="E344" s="146">
+        <v>239</v>
+      </c>
+      <c r="F344" s="146">
+        <v>250</v>
+      </c>
       <c r="G344" s="146"/>
       <c r="H344" s="147"/>
     </row>
-    <row r="345" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B345" s="149"/>
-      <c r="C345" s="145"/>
+    <row r="345" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A345" s="116" t="str">
+        <f>LEFT(B345, FIND("-", B345) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B345" s="116" t="inlineStr">
+        <is>
+          <t>PROS-PERMITNUM</t>
+        </is>
+      </c>
+      <c r="C345" s="145" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="D345" s="146"/>
-      <c r="E345" s="146"/>
-      <c r="F345" s="146"/>
+      <c r="E345" s="146">
+        <v>171</v>
+      </c>
+      <c r="F345" s="146">
+        <v>240</v>
+      </c>
       <c r="G345" s="146"/>
       <c r="H345" s="147"/>
     </row>
-    <row r="346" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B346" s="149"/>
-      <c r="C346" s="145"/>
+    <row r="346" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A346" s="116" t="str">
+        <f>LEFT(B346, FIND("-", B346) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B346" s="116" t="inlineStr">
+        <is>
+          <t>PROS-PERMITNUM</t>
+        </is>
+      </c>
+      <c r="C346" s="145" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="D346" s="146"/>
-      <c r="E346" s="146"/>
-      <c r="F346" s="146"/>
+      <c r="E346" s="146">
+        <v>221</v>
+      </c>
+      <c r="F346" s="146">
+        <v>240</v>
+      </c>
       <c r="G346" s="146"/>
       <c r="H346" s="147"/>
     </row>
-    <row r="347" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B347" s="149"/>
-      <c r="C347" s="145"/>
+    <row r="347" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A347" s="116" t="str">
+        <f>LEFT(B347, FIND("-", B347) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B347" s="116" t="inlineStr">
+        <is>
+          <t>PROS-PERMITNUM</t>
+        </is>
+      </c>
+      <c r="C347" s="145" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="D347" s="146"/>
-      <c r="E347" s="146"/>
-      <c r="F347" s="146"/>
+      <c r="E347" s="146">
+        <v>242</v>
+      </c>
+      <c r="F347" s="146">
+        <v>240</v>
+      </c>
       <c r="G347" s="146"/>
       <c r="H347" s="147"/>
     </row>
-    <row r="348" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B348" s="149"/>
-      <c r="C348" s="145"/>
+    <row r="348" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A348" s="116" t="str">
+        <f>LEFT(B348, FIND("-", B348) - 1)</f>
+        <v>PROS</v>
+      </c>
+      <c r="B348" s="116" t="inlineStr">
+        <is>
+          <t>PROS-PERMITNUM</t>
+        </is>
+      </c>
+      <c r="C348" s="145" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="D348" s="146"/>
-      <c r="E348" s="146"/>
-      <c r="F348" s="146"/>
+      <c r="E348" s="146">
+        <v>239</v>
+      </c>
+      <c r="F348" s="146">
+        <v>240</v>
+      </c>
       <c r="G348" s="146"/>
       <c r="H348" s="147"/>
     </row>

</xml_diff>